<commit_message>
Corrected the eye center finding formula
</commit_message>
<xml_diff>
--- a/eye_detection_results.xlsx
+++ b/eye_detection_results.xlsx
@@ -723,304 +723,304 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>440.3939329852715</v>
+        <v>1023.206486448264</v>
       </c>
       <c r="C2" t="n">
-        <v>501.5137479855144</v>
+        <v>1035.466708121946</v>
       </c>
       <c r="D2" t="n">
-        <v>462.2932871336475</v>
+        <v>1027.393110137574</v>
       </c>
       <c r="E2" t="n">
-        <v>503.6644353313861</v>
+        <v>1035.460130476199</v>
       </c>
       <c r="F2" t="n">
-        <v>509.8228039020467</v>
+        <v>1029.29412657916</v>
       </c>
       <c r="G2" t="n">
-        <v>511.9224736783108</v>
+        <v>1033.749379085888</v>
       </c>
       <c r="H2" t="n">
-        <v>492.5389178048484</v>
+        <v>1038.780658430179</v>
       </c>
       <c r="I2" t="n">
-        <v>505.3427774656331</v>
+        <v>1036.841188293242</v>
       </c>
       <c r="J2" t="n">
-        <v>500.2602588189607</v>
+        <v>1041.377405217012</v>
       </c>
       <c r="K2" t="n">
-        <v>502.5765111329859</v>
+        <v>1028.567567878164</v>
       </c>
       <c r="L2" t="n">
-        <v>490.8120615766293</v>
+        <v>1033.306448213499</v>
       </c>
       <c r="M2" t="n">
-        <v>495.080287761631</v>
+        <v>1037.238602067875</v>
       </c>
       <c r="N2" t="n">
-        <v>503.4634148254538</v>
+        <v>1043.229365646232</v>
       </c>
       <c r="O2" t="n">
-        <v>496.9347824132035</v>
+        <v>1036.57776402562</v>
       </c>
       <c r="P2" t="n">
-        <v>494.4297923002397</v>
+        <v>1042.738599925124</v>
       </c>
       <c r="Q2" t="n">
-        <v>493.9171970918829</v>
+        <v>1033.159265162856</v>
       </c>
       <c r="R2" t="n">
-        <v>515.7511149992484</v>
+        <v>1036.947435844322</v>
       </c>
       <c r="S2" t="n">
-        <v>479.7471116868115</v>
+        <v>1036.579781140423</v>
       </c>
       <c r="T2" t="n">
-        <v>500.8866447221948</v>
+        <v>1038.26740678304</v>
       </c>
       <c r="U2" t="n">
-        <v>501.7556670664812</v>
+        <v>1033.822047074477</v>
       </c>
       <c r="V2" t="n">
-        <v>540.4103153458225</v>
+        <v>1040.835562592596</v>
       </c>
       <c r="W2" t="n">
-        <v>505.7783546260189</v>
+        <v>1042.286114988325</v>
       </c>
       <c r="X2" t="n">
-        <v>495.1863721473616</v>
+        <v>1045.179496815958</v>
       </c>
       <c r="Y2" t="n">
-        <v>471.1006915782591</v>
+        <v>1041.166341368316</v>
       </c>
       <c r="Z2" t="n">
-        <v>460.1357947251067</v>
+        <v>1041.846556814554</v>
       </c>
       <c r="AA2" t="n">
-        <v>465.1704196713624</v>
+        <v>1041.410164199395</v>
       </c>
       <c r="AB2" t="n">
-        <v>493.4914963366977</v>
+        <v>1042.068895244689</v>
       </c>
       <c r="AC2" t="n">
-        <v>488.8833519414849</v>
+        <v>1044.340465187395</v>
       </c>
       <c r="AD2" t="n">
-        <v>506.8068935555506</v>
+        <v>1041.754017763988</v>
       </c>
       <c r="AE2" t="n">
-        <v>499.2370718998854</v>
+        <v>1040.087204286211</v>
       </c>
       <c r="AF2" t="n">
-        <v>498.3104247761286</v>
+        <v>1040.166518508974</v>
       </c>
       <c r="AG2" t="n">
-        <v>504.6416072041148</v>
+        <v>1047.710598318946</v>
       </c>
       <c r="AH2" t="n">
-        <v>448.6866598826644</v>
+        <v>1039.435967982753</v>
       </c>
       <c r="AI2" t="n">
-        <v>499.8039469215612</v>
+        <v>1042.615671277115</v>
       </c>
       <c r="AJ2" t="n">
-        <v>503.5768792932276</v>
+        <v>1038.55767754319</v>
       </c>
       <c r="AK2" t="n">
-        <v>464.7812632570997</v>
+        <v>1040.498416344626</v>
       </c>
       <c r="AL2" t="n">
-        <v>537.213341704536</v>
+        <v>1042.997746283471</v>
       </c>
       <c r="AM2" t="n">
-        <v>507.8844864187662</v>
+        <v>1040.998880255194</v>
       </c>
       <c r="AN2" t="n">
-        <v>503.6412243684878</v>
+        <v>1042.129258902628</v>
       </c>
       <c r="AO2" t="n">
-        <v>500.7276892480615</v>
+        <v>1042.524459780986</v>
       </c>
       <c r="AP2" t="n">
-        <v>497.7308233945123</v>
+        <v>1041.306867497145</v>
       </c>
       <c r="AQ2" t="n">
-        <v>466.1183628934979</v>
+        <v>1039.183528533651</v>
       </c>
       <c r="AR2" t="n">
-        <v>494.6865504391998</v>
+        <v>1034.691926969352</v>
       </c>
       <c r="AS2" t="n">
-        <v>554.4429396781112</v>
+        <v>1035.504238646513</v>
       </c>
       <c r="AT2" t="n">
-        <v>386.0008558115597</v>
+        <v>1040.692758667571</v>
       </c>
       <c r="AU2" t="n">
-        <v>535.4658215553851</v>
+        <v>1034.236384779125</v>
       </c>
       <c r="AV2" t="n">
-        <v>496.2994105877941</v>
+        <v>1038.591258557645</v>
       </c>
       <c r="AW2" t="n">
-        <v>503.1471133281842</v>
+        <v>1031.857510950081</v>
       </c>
       <c r="AX2" t="n">
-        <v>448.8469343851077</v>
+        <v>1037.681842987879</v>
       </c>
       <c r="AY2" t="n">
-        <v>522.434458373082</v>
+        <v>1035.56217695338</v>
       </c>
       <c r="AZ2" t="n">
-        <v>505.601888301189</v>
+        <v>1042.770817059139</v>
       </c>
       <c r="BA2" t="n">
-        <v>497.6619147998733</v>
+        <v>978.7827426274629</v>
       </c>
       <c r="BB2" t="n">
-        <v>499.4552507336103</v>
+        <v>1041.327104205305</v>
       </c>
       <c r="BC2" t="n">
-        <v>457.3209442396877</v>
+        <v>1039.146795663856</v>
       </c>
       <c r="BD2" t="n">
-        <v>495.2365562024249</v>
+        <v>1048.008810306915</v>
       </c>
       <c r="BE2" t="n">
-        <v>474.1980388661388</v>
+        <v>1040.463336636799</v>
       </c>
       <c r="BF2" t="n">
-        <v>484.2381702463962</v>
+        <v>1045.688225920134</v>
       </c>
       <c r="BG2" t="n">
-        <v>515.9179529220033</v>
+        <v>1038.242049969467</v>
       </c>
       <c r="BH2" t="n">
-        <v>538.7538051543761</v>
+        <v>1039.703543098643</v>
       </c>
       <c r="BI2" t="n">
-        <v>531.85388071095</v>
+        <v>1041.121832235701</v>
       </c>
       <c r="BJ2" t="n">
-        <v>498.0678534306277</v>
+        <v>1041.202501059864</v>
       </c>
       <c r="BK2" t="n">
-        <v>500.3139151306328</v>
+        <v>1040.676330381689</v>
       </c>
       <c r="BL2" t="n">
-        <v>495.8955717829919</v>
+        <v>1035.410240792355</v>
       </c>
       <c r="BM2" t="n">
-        <v>463.0536200296276</v>
+        <v>982.6187396178384</v>
       </c>
       <c r="BN2" t="n">
-        <v>470.9079808802786</v>
+        <v>1039.547473073163</v>
       </c>
       <c r="BO2" t="n">
-        <v>437.2452886745482</v>
+        <v>1040.61657378551</v>
       </c>
       <c r="BP2" t="n">
-        <v>434.6415940279138</v>
+        <v>980.5323608028235</v>
       </c>
       <c r="BQ2" t="n">
-        <v>509.0534248339184</v>
+        <v>1042.813295880913</v>
       </c>
       <c r="BR2" t="n">
-        <v>428.5008736291434</v>
+        <v>988.5903416813984</v>
       </c>
       <c r="BS2" t="n">
-        <v>470.2207060995493</v>
+        <v>1037.652304230957</v>
       </c>
       <c r="BT2" t="n">
-        <v>272.6628768712395</v>
+        <v>1042.267133285329</v>
       </c>
       <c r="BU2" t="n">
-        <v>532.200388960985</v>
+        <v>1030.953069158405</v>
       </c>
       <c r="BV2" t="n">
-        <v>465.0091644684435</v>
+        <v>1037.035416809226</v>
       </c>
       <c r="BW2" t="n">
-        <v>553.6669500726869</v>
+        <v>984.8671032572611</v>
       </c>
       <c r="BX2" t="n">
-        <v>515.7860288249185</v>
+        <v>984.7548529809719</v>
       </c>
       <c r="BY2" t="n">
-        <v>555.6754056464983</v>
+        <v>1039.781321871812</v>
       </c>
       <c r="BZ2" t="n">
-        <v>493.2250019775241</v>
+        <v>1040.693395018523</v>
       </c>
       <c r="CA2" t="n">
-        <v>502.8236766859898</v>
+        <v>980.3866093963645</v>
       </c>
       <c r="CB2" t="n">
-        <v>509.240227959029</v>
+        <v>983.048553046862</v>
       </c>
       <c r="CC2" t="n">
-        <v>493.6308471928337</v>
+        <v>1036.765944612191</v>
       </c>
       <c r="CD2" t="n">
-        <v>501.9433027158534</v>
+        <v>1038.376848930385</v>
       </c>
       <c r="CE2" t="n">
-        <v>431.8123790981648</v>
+        <v>1045.055434281791</v>
       </c>
       <c r="CF2" t="n">
-        <v>489.0018031278172</v>
+        <v>943.1175040664518</v>
       </c>
       <c r="CG2" t="n">
-        <v>450.611385607234</v>
+        <v>938.0990584553132</v>
       </c>
       <c r="CH2" t="n">
-        <v>477.5306567663687</v>
+        <v>982.795424563645</v>
       </c>
       <c r="CI2" t="n">
-        <v>452.8336344005464</v>
+        <v>1041.552896895669</v>
       </c>
       <c r="CJ2" t="n">
-        <v>520.5128330691523</v>
+        <v>1041.149388453517</v>
       </c>
       <c r="CK2" t="n">
-        <v>533.2125383851821</v>
+        <v>982.1528455512671</v>
       </c>
       <c r="CL2" t="n">
-        <v>451.2174389873604</v>
+        <v>977.2506307117088</v>
       </c>
       <c r="CM2" t="n">
-        <v>421.4990583559599</v>
+        <v>934.8830256902256</v>
       </c>
       <c r="CN2" t="n">
-        <v>519.7367929907737</v>
+        <v>935.6784490209317</v>
       </c>
       <c r="CO2" t="n">
-        <v>386.9928732080399</v>
+        <v>979.6501317316936</v>
       </c>
       <c r="CP2" t="n">
-        <v>417.5758689996144</v>
+        <v>977.5574164378777</v>
       </c>
       <c r="CQ2" t="n">
-        <v>330.7363613030374</v>
+        <v>1041.380194343776</v>
       </c>
       <c r="CR2" t="n">
-        <v>382.8105203001904</v>
+        <v>983.2656217348688</v>
       </c>
       <c r="CS2" t="n">
-        <v>329.8856448745266</v>
+        <v>977.7974827573231</v>
       </c>
       <c r="CT2" t="n">
-        <v>528.1761371985355</v>
+        <v>935.888729306226</v>
       </c>
       <c r="CU2" t="n">
-        <v>486.2668834612356</v>
+        <v>977.4880863251565</v>
       </c>
       <c r="CV2" t="n">
-        <v>444.3009323105604</v>
+        <v>976.6397482240442</v>
       </c>
       <c r="CW2" t="n">
-        <v>485.8350997660682</v>
+        <v>1041.052837933324</v>
       </c>
     </row>
     <row r="3">
@@ -1028,304 +1028,304 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>460.0170901382378</v>
+        <v>1027.343936206536</v>
       </c>
       <c r="C3" t="n">
-        <v>479.6805426598306</v>
+        <v>1032.578762712718</v>
       </c>
       <c r="D3" t="n">
-        <v>495.341682135705</v>
+        <v>1039.396020581187</v>
       </c>
       <c r="E3" t="n">
-        <v>493.3116352945346</v>
+        <v>1041.671904073432</v>
       </c>
       <c r="F3" t="n">
-        <v>509.8228039020467</v>
+        <v>1037.29580769522</v>
       </c>
       <c r="G3" t="n">
-        <v>511.9224736783108</v>
+        <v>1037.098199646513</v>
       </c>
       <c r="H3" t="n">
-        <v>492.5389178048484</v>
+        <v>1046.417799665617</v>
       </c>
       <c r="I3" t="n">
-        <v>505.3427774656331</v>
+        <v>1041.573431906017</v>
       </c>
       <c r="J3" t="n">
-        <v>500.2602588189607</v>
+        <v>1043.028172437884</v>
       </c>
       <c r="K3" t="n">
-        <v>502.5765111329859</v>
+        <v>1041.070217982987</v>
       </c>
       <c r="L3" t="n">
-        <v>501.9256239066611</v>
+        <v>1033.306448213499</v>
       </c>
       <c r="M3" t="n">
-        <v>495.080287761631</v>
+        <v>1037.238602067875</v>
       </c>
       <c r="N3" t="n">
-        <v>503.4634148254538</v>
+        <v>1043.229365646232</v>
       </c>
       <c r="O3" t="n">
-        <v>499.8330746778271</v>
+        <v>1036.57776402562</v>
       </c>
       <c r="P3" t="n">
-        <v>494.4297923002397</v>
+        <v>1042.738599925124</v>
       </c>
       <c r="Q3" t="n">
-        <v>503.9232918477925</v>
+        <v>1033.159265162856</v>
       </c>
       <c r="R3" t="n">
-        <v>504.8887750880898</v>
+        <v>1036.947435844322</v>
       </c>
       <c r="S3" t="n">
-        <v>499.7845302963906</v>
+        <v>1036.579781140423</v>
       </c>
       <c r="T3" t="n">
-        <v>502.3993993840437</v>
+        <v>1042.773665453914</v>
       </c>
       <c r="U3" t="n">
-        <v>501.7556670664812</v>
+        <v>1033.822047074477</v>
       </c>
       <c r="V3" t="n">
-        <v>540.4103153458225</v>
+        <v>1040.835562592596</v>
       </c>
       <c r="W3" t="n">
-        <v>505.7783546260189</v>
+        <v>1042.286114988325</v>
       </c>
       <c r="X3" t="n">
-        <v>495.1863721473616</v>
+        <v>1045.179496815958</v>
       </c>
       <c r="Y3" t="n">
-        <v>453.5461909144649</v>
+        <v>1042.662793665702</v>
       </c>
       <c r="Z3" t="n">
-        <v>460.1357947251067</v>
+        <v>1047.325972633274</v>
       </c>
       <c r="AA3" t="n">
-        <v>465.1704196713624</v>
+        <v>1042.839415833603</v>
       </c>
       <c r="AB3" t="n">
-        <v>465.3010655102863</v>
+        <v>1042.068895244689</v>
       </c>
       <c r="AC3" t="n">
-        <v>488.8833519414849</v>
+        <v>1044.340465187395</v>
       </c>
       <c r="AD3" t="n">
-        <v>506.8068935555506</v>
+        <v>1041.754017763988</v>
       </c>
       <c r="AE3" t="n">
-        <v>460.3088863663555</v>
+        <v>1044.845801153267</v>
       </c>
       <c r="AF3" t="n">
-        <v>455.0005679236029</v>
+        <v>1040.166518508974</v>
       </c>
       <c r="AG3" t="n">
-        <v>504.6416072041148</v>
+        <v>1043.025102085961</v>
       </c>
       <c r="AH3" t="n">
-        <v>429.794701708568</v>
+        <v>1039.435967982753</v>
       </c>
       <c r="AI3" t="n">
-        <v>499.8039469215612</v>
+        <v>1042.615671277115</v>
       </c>
       <c r="AJ3" t="n">
-        <v>503.5768792932276</v>
+        <v>1042.941225355646</v>
       </c>
       <c r="AK3" t="n">
-        <v>444.2141586762804</v>
+        <v>1040.498416344626</v>
       </c>
       <c r="AL3" t="n">
-        <v>507.031804015506</v>
+        <v>1042.997746283471</v>
       </c>
       <c r="AM3" t="n">
-        <v>507.8844864187662</v>
+        <v>1040.998880255194</v>
       </c>
       <c r="AN3" t="n">
-        <v>503.6412243684878</v>
+        <v>1042.129258902628</v>
       </c>
       <c r="AO3" t="n">
-        <v>500.7276892480615</v>
+        <v>1042.524459780986</v>
       </c>
       <c r="AP3" t="n">
-        <v>540.1755433505789</v>
+        <v>981.0156209132829</v>
       </c>
       <c r="AQ3" t="n">
-        <v>441.685116934714</v>
+        <v>1041.152004783439</v>
       </c>
       <c r="AR3" t="n">
-        <v>466.8343408184446</v>
+        <v>972.1847620192463</v>
       </c>
       <c r="AS3" t="n">
-        <v>537.9680290917877</v>
+        <v>1038.049759662988</v>
       </c>
       <c r="AT3" t="n">
-        <v>490.7088166967895</v>
+        <v>1040.692758667571</v>
       </c>
       <c r="AU3" t="n">
-        <v>535.4658215553851</v>
+        <v>1034.236384779125</v>
       </c>
       <c r="AV3" t="n">
-        <v>496.2994105877941</v>
+        <v>1038.591258557645</v>
       </c>
       <c r="AW3" t="n">
-        <v>468.3721130940546</v>
+        <v>935.5386014568634</v>
       </c>
       <c r="AX3" t="n">
-        <v>440.8197532082397</v>
+        <v>1037.681842987879</v>
       </c>
       <c r="AY3" t="n">
-        <v>460.7089235249878</v>
+        <v>1035.56217695338</v>
       </c>
       <c r="AZ3" t="n">
-        <v>505.601888301189</v>
+        <v>975.1777704629455</v>
       </c>
       <c r="BA3" t="n">
-        <v>505.0087835937373</v>
+        <v>978.7827426274629</v>
       </c>
       <c r="BB3" t="n">
-        <v>499.4552507336103</v>
+        <v>1033.757028489714</v>
       </c>
       <c r="BC3" t="n">
-        <v>457.3209442396877</v>
+        <v>1039.146795663856</v>
       </c>
       <c r="BD3" t="n">
-        <v>456.4702073632367</v>
+        <v>1037.562653575351</v>
       </c>
       <c r="BE3" t="n">
-        <v>482.6068100538958</v>
+        <v>977.4627116398508</v>
       </c>
       <c r="BF3" t="n">
-        <v>444.1590374559729</v>
+        <v>985.5525160284876</v>
       </c>
       <c r="BG3" t="n">
-        <v>510.5485442788951</v>
+        <v>1038.242049969467</v>
       </c>
       <c r="BH3" t="n">
-        <v>505.4880580329894</v>
+        <v>977.0125315754669</v>
       </c>
       <c r="BI3" t="n">
-        <v>499.7174844629693</v>
+        <v>1037.720443614627</v>
       </c>
       <c r="BJ3" t="n">
-        <v>472.2102660482882</v>
+        <v>1036.936034655617</v>
       </c>
       <c r="BK3" t="n">
-        <v>433.0964102483513</v>
+        <v>1040.676330381689</v>
       </c>
       <c r="BL3" t="n">
-        <v>450.576515412537</v>
+        <v>1035.410240792355</v>
       </c>
       <c r="BM3" t="n">
-        <v>445.6508688163742</v>
+        <v>982.6187396178384</v>
       </c>
       <c r="BN3" t="n">
-        <v>431.3522284465912</v>
+        <v>1041.124591615898</v>
       </c>
       <c r="BO3" t="n">
-        <v>425.1918408541445</v>
+        <v>1040.61657378551</v>
       </c>
       <c r="BP3" t="n">
-        <v>403.8761779890831</v>
+        <v>980.5323608028235</v>
       </c>
       <c r="BQ3" t="n">
-        <v>497.2352377918311</v>
+        <v>940.7476914931907</v>
       </c>
       <c r="BR3" t="n">
-        <v>288.803175867375</v>
+        <v>985.888990576734</v>
       </c>
       <c r="BS3" t="n">
-        <v>453.1834076426829</v>
+        <v>976.5931895675516</v>
       </c>
       <c r="BT3" t="n">
-        <v>233.5780148919479</v>
+        <v>984.5896248174329</v>
       </c>
       <c r="BU3" t="n">
-        <v>505.2447097526381</v>
+        <v>1038.868950724653</v>
       </c>
       <c r="BV3" t="n">
-        <v>465.0091644684435</v>
+        <v>1041.054023624978</v>
       </c>
       <c r="BW3" t="n">
-        <v>521.6500983148345</v>
+        <v>983.4635213207359</v>
       </c>
       <c r="BX3" t="n">
-        <v>495.8900962063441</v>
+        <v>940.655739907653</v>
       </c>
       <c r="BY3" t="n">
-        <v>512.0622909827584</v>
+        <v>980.529634267112</v>
       </c>
       <c r="BZ3" t="n">
-        <v>467.3147344203259</v>
+        <v>935.6138356788564</v>
       </c>
       <c r="CA3" t="n">
-        <v>502.8236766859898</v>
+        <v>936.2989170624248</v>
       </c>
       <c r="CB3" t="n">
-        <v>487.1954346208366</v>
+        <v>938.4651130713622</v>
       </c>
       <c r="CC3" t="n">
-        <v>463.2518335053386</v>
+        <v>940.3661615396155</v>
       </c>
       <c r="CD3" t="n">
-        <v>457.9545259517413</v>
+        <v>1038.376848930385</v>
       </c>
       <c r="CE3" t="n">
-        <v>431.8123790981648</v>
+        <v>1045.055434281791</v>
       </c>
       <c r="CF3" t="n">
-        <v>489.0018031278172</v>
+        <v>943.1175040664518</v>
       </c>
       <c r="CG3" t="n">
-        <v>450.611385607234</v>
+        <v>938.0990584553132</v>
       </c>
       <c r="CH3" t="n">
-        <v>445.1791313171462</v>
+        <v>979.3176802567308</v>
       </c>
       <c r="CI3" t="n">
-        <v>429.0556816238906</v>
+        <v>979.9882936577256</v>
       </c>
       <c r="CJ3" t="n">
-        <v>379.0870553796667</v>
+        <v>938.4400311475525</v>
       </c>
       <c r="CK3" t="n">
-        <v>489.3500264482186</v>
+        <v>982.7922904237206</v>
       </c>
       <c r="CL3" t="n">
-        <v>445.8094361783722</v>
+        <v>932.8387295087239</v>
       </c>
       <c r="CM3" t="n">
-        <v>364.1389972489948</v>
+        <v>935.6830256902256</v>
       </c>
       <c r="CN3" t="n">
-        <v>378.9888909102517</v>
+        <v>935.6784490209317</v>
       </c>
       <c r="CO3" t="n">
-        <v>363.0799939481722</v>
+        <v>938.1190842487076</v>
       </c>
       <c r="CP3" t="n">
-        <v>358.4046141807215</v>
+        <v>935.8563625867139</v>
       </c>
       <c r="CQ3" t="n">
-        <v>329.39016991313</v>
+        <v>938.1492994753349</v>
       </c>
       <c r="CR3" t="n">
-        <v>269.0270393139573</v>
+        <v>935.653764269982</v>
       </c>
       <c r="CS3" t="n">
-        <v>329.8856448745266</v>
+        <v>935.7666798366245</v>
       </c>
       <c r="CT3" t="n">
-        <v>473.5149479351156</v>
+        <v>935.888729306226</v>
       </c>
       <c r="CU3" t="n">
-        <v>486.2668834612356</v>
+        <v>935.5373005349059</v>
       </c>
       <c r="CV3" t="n">
-        <v>444.3009323105604</v>
+        <v>976.6397482240442</v>
       </c>
       <c r="CW3" t="n">
-        <v>484.2221137358345</v>
+        <v>1037.45144931225</v>
       </c>
     </row>
     <row r="4">
@@ -1333,304 +1333,304 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>460.0170901382378</v>
+        <v>1027.343936206536</v>
       </c>
       <c r="C4" t="n">
-        <v>481.2029200620591</v>
+        <v>1032.578762712718</v>
       </c>
       <c r="D4" t="n">
-        <v>495.341682135705</v>
+        <v>1039.396020581187</v>
       </c>
       <c r="E4" t="n">
-        <v>493.3116352945346</v>
+        <v>1041.671904073432</v>
       </c>
       <c r="F4" t="n">
-        <v>509.8228039020467</v>
+        <v>1037.29580769522</v>
       </c>
       <c r="G4" t="n">
-        <v>492.8398027523702</v>
+        <v>1037.098199646513</v>
       </c>
       <c r="H4" t="n">
-        <v>492.5389178048484</v>
+        <v>1046.417799665617</v>
       </c>
       <c r="I4" t="n">
-        <v>505.3427774656331</v>
+        <v>1042.969700821223</v>
       </c>
       <c r="J4" t="n">
-        <v>500.2602588189607</v>
+        <v>1043.028172437884</v>
       </c>
       <c r="K4" t="n">
-        <v>502.5765111329859</v>
+        <v>1041.070217982987</v>
       </c>
       <c r="L4" t="n">
-        <v>501.9256239066611</v>
+        <v>1033.306448213499</v>
       </c>
       <c r="M4" t="n">
-        <v>493.9963849711586</v>
+        <v>1037.238602067875</v>
       </c>
       <c r="N4" t="n">
-        <v>494.7002537074298</v>
+        <v>1043.229365646232</v>
       </c>
       <c r="O4" t="n">
-        <v>499.8330746778271</v>
+        <v>1041.505291053368</v>
       </c>
       <c r="P4" t="n">
-        <v>494.4297923002397</v>
+        <v>1042.738599925124</v>
       </c>
       <c r="Q4" t="n">
-        <v>504.0619404445785</v>
+        <v>1038.709162180021</v>
       </c>
       <c r="R4" t="n">
-        <v>504.8887750880898</v>
+        <v>1041.710310523521</v>
       </c>
       <c r="S4" t="n">
-        <v>499.7845302963906</v>
+        <v>1044.369966634909</v>
       </c>
       <c r="T4" t="n">
-        <v>462.2653502276574</v>
+        <v>1043.449968536461</v>
       </c>
       <c r="U4" t="n">
-        <v>501.7556670664812</v>
+        <v>1010.605657049498</v>
       </c>
       <c r="V4" t="n">
-        <v>540.4103153458225</v>
+        <v>1017.569141583906</v>
       </c>
       <c r="W4" t="n">
-        <v>463.0072886159591</v>
+        <v>1042.286114988325</v>
       </c>
       <c r="X4" t="n">
-        <v>495.1863721473616</v>
+        <v>962.7198164025173</v>
       </c>
       <c r="Y4" t="n">
-        <v>453.5461909144649</v>
+        <v>1041.166341368316</v>
       </c>
       <c r="Z4" t="n">
-        <v>441.1267342773996</v>
+        <v>957.7896855996969</v>
       </c>
       <c r="AA4" t="n">
-        <v>465.1704196713624</v>
+        <v>1018.521488787138</v>
       </c>
       <c r="AB4" t="n">
-        <v>465.3010655102863</v>
+        <v>1042.068895244689</v>
       </c>
       <c r="AC4" t="n">
-        <v>499.5255322930675</v>
+        <v>1020.100510397404</v>
       </c>
       <c r="AD4" t="n">
-        <v>506.8068935555506</v>
+        <v>1017.497227950182</v>
       </c>
       <c r="AE4" t="n">
-        <v>460.3088863663555</v>
+        <v>913.2955360925804</v>
       </c>
       <c r="AF4" t="n">
-        <v>470.392314047767</v>
+        <v>996.9461694551086</v>
       </c>
       <c r="AG4" t="n">
-        <v>504.6416072041148</v>
+        <v>915.6570789520061</v>
       </c>
       <c r="AH4" t="n">
-        <v>436.2829803895678</v>
+        <v>995.7296857575257</v>
       </c>
       <c r="AI4" t="n">
-        <v>459.233438279675</v>
+        <v>999.3953222232491</v>
       </c>
       <c r="AJ4" t="n">
-        <v>503.5768792932276</v>
+        <v>895.2913640863659</v>
       </c>
       <c r="AK4" t="n">
-        <v>444.2141586762804</v>
+        <v>997.2780672907604</v>
       </c>
       <c r="AL4" t="n">
-        <v>507.031804015506</v>
+        <v>999.7773972296051</v>
       </c>
       <c r="AM4" t="n">
-        <v>507.8844864187662</v>
+        <v>997.7785312013282</v>
       </c>
       <c r="AN4" t="n">
-        <v>491.2158321311705</v>
+        <v>939.3101719171455</v>
       </c>
       <c r="AO4" t="n">
-        <v>499.1822153084308</v>
+        <v>1015.00421667892</v>
       </c>
       <c r="AP4" t="n">
-        <v>491.9343169389867</v>
+        <v>935.1897205839532</v>
       </c>
       <c r="AQ4" t="n">
-        <v>441.685116934714</v>
+        <v>997.9316557295728</v>
       </c>
       <c r="AR4" t="n">
-        <v>461.1304240528516</v>
+        <v>926.462984685378</v>
       </c>
       <c r="AS4" t="n">
-        <v>537.9680290917877</v>
+        <v>994.829410609122</v>
       </c>
       <c r="AT4" t="n">
-        <v>490.7088166967895</v>
+        <v>939.3646267082364</v>
       </c>
       <c r="AU4" t="n">
-        <v>526.2239762478387</v>
+        <v>936.7685002748146</v>
       </c>
       <c r="AV4" t="n">
-        <v>457.4976830599802</v>
+        <v>995.3709095037788</v>
       </c>
       <c r="AW4" t="n">
-        <v>468.3721130940546</v>
+        <v>892.3182524029977</v>
       </c>
       <c r="AX4" t="n">
-        <v>440.8197532082397</v>
+        <v>933.74570002447</v>
       </c>
       <c r="AY4" t="n">
-        <v>460.7089235249878</v>
+        <v>934.3079393269329</v>
       </c>
       <c r="AZ4" t="n">
-        <v>485.6442524612379</v>
+        <v>897.1721777866421</v>
       </c>
       <c r="BA4" t="n">
-        <v>461.5408995252598</v>
+        <v>936.4209722173598</v>
       </c>
       <c r="BB4" t="n">
-        <v>499.4552507336103</v>
+        <v>998.1067551514388</v>
       </c>
       <c r="BC4" t="n">
-        <v>457.3209442396877</v>
+        <v>995.9264466099906</v>
       </c>
       <c r="BD4" t="n">
-        <v>322.5359337888919</v>
+        <v>994.3423045214855</v>
       </c>
       <c r="BE4" t="n">
-        <v>361.9615757347714</v>
+        <v>931.6409739649113</v>
       </c>
       <c r="BF4" t="n">
-        <v>419.0886293587333</v>
+        <v>894.9123322864891</v>
       </c>
       <c r="BG4" t="n">
-        <v>504.9933936322662</v>
+        <v>992.6084912824263</v>
       </c>
       <c r="BH4" t="n">
-        <v>493.6438447777865</v>
+        <v>933.7921825216011</v>
       </c>
       <c r="BI4" t="n">
-        <v>464.9838627600693</v>
+        <v>994.5000945607611</v>
       </c>
       <c r="BJ4" t="n">
-        <v>472.2102660482882</v>
+        <v>933.8621598567195</v>
       </c>
       <c r="BK4" t="n">
-        <v>433.0964102483513</v>
+        <v>997.4559813278231</v>
       </c>
       <c r="BL4" t="n">
-        <v>429.2186192898953</v>
+        <v>994.6955306331784</v>
       </c>
       <c r="BM4" t="n">
-        <v>414.2988794232926</v>
+        <v>939.3983905639727</v>
       </c>
       <c r="BN4" t="n">
-        <v>431.3522284465912</v>
+        <v>937.2282053044155</v>
       </c>
       <c r="BO4" t="n">
-        <v>425.1918408541445</v>
+        <v>997.3962247316443</v>
       </c>
       <c r="BP4" t="n">
-        <v>403.8761779890831</v>
+        <v>937.3120117489576</v>
       </c>
       <c r="BQ4" t="n">
-        <v>345.5570423793334</v>
+        <v>897.527342439325</v>
       </c>
       <c r="BR4" t="n">
-        <v>277.4561114389369</v>
+        <v>897.7364088316524</v>
       </c>
       <c r="BS4" t="n">
-        <v>339.2449458468159</v>
+        <v>891.6959146637607</v>
       </c>
       <c r="BT4" t="n">
-        <v>211.6359138547718</v>
+        <v>897.2701626902483</v>
       </c>
       <c r="BU4" t="n">
-        <v>481.5915152334688</v>
+        <v>892.0773893946209</v>
       </c>
       <c r="BV4" t="n">
-        <v>465.0091644684435</v>
+        <v>893.8254197831648</v>
       </c>
       <c r="BW4" t="n">
-        <v>493.4346433590889</v>
+        <v>892.5938738126672</v>
       </c>
       <c r="BX4" t="n">
-        <v>490.409162631619</v>
+        <v>894.9353908537872</v>
       </c>
       <c r="BY4" t="n">
-        <v>506.5252809628793</v>
+        <v>934.7037339377823</v>
       </c>
       <c r="BZ4" t="n">
-        <v>462.5776063807463</v>
+        <v>893.1934866249907</v>
       </c>
       <c r="CA4" t="n">
-        <v>465.0824892604251</v>
+        <v>893.0785680085592</v>
       </c>
       <c r="CB4" t="n">
-        <v>464.1273430115328</v>
+        <v>892.8432937471574</v>
       </c>
       <c r="CC4" t="n">
-        <v>434.8595291762122</v>
+        <v>894.7443422154108</v>
       </c>
       <c r="CD4" t="n">
-        <v>434.9473068886006</v>
+        <v>937.8923985008948</v>
       </c>
       <c r="CE4" t="n">
-        <v>431.8123790981648</v>
+        <v>897.8200617984861</v>
       </c>
       <c r="CF4" t="n">
-        <v>432.0583810769822</v>
+        <v>897.7955425287319</v>
       </c>
       <c r="CG4" t="n">
-        <v>431.447556605777</v>
+        <v>894.8787094014473</v>
       </c>
       <c r="CH4" t="n">
-        <v>441.3026571810516</v>
+        <v>936.873724405115</v>
       </c>
       <c r="CI4" t="n">
-        <v>429.0556816238906</v>
+        <v>936.7679446038599</v>
       </c>
       <c r="CJ4" t="n">
-        <v>379.0870553796667</v>
+        <v>895.2196820936867</v>
       </c>
       <c r="CK4" t="n">
-        <v>469.023517122968</v>
+        <v>894.8132263529317</v>
       </c>
       <c r="CL4" t="n">
-        <v>331.6488526439006</v>
+        <v>889.6183804548582</v>
       </c>
       <c r="CM4" t="n">
-        <v>364.1389972489948</v>
+        <v>892.4626766363599</v>
       </c>
       <c r="CN4" t="n">
-        <v>359.5259976641831</v>
+        <v>892.4580999670659</v>
       </c>
       <c r="CO4" t="n">
-        <v>271.8148867840877</v>
+        <v>894.8987351948419</v>
       </c>
       <c r="CP4" t="n">
-        <v>358.4046141807215</v>
+        <v>892.6360135328481</v>
       </c>
       <c r="CQ4" t="n">
-        <v>287.3769183105074</v>
+        <v>894.9289504214692</v>
       </c>
       <c r="CR4" t="n">
-        <v>269.0270393139573</v>
+        <v>892.4334152161164</v>
       </c>
       <c r="CS4" t="n">
-        <v>329.8856448745266</v>
+        <v>892.5463307827588</v>
       </c>
       <c r="CT4" t="n">
-        <v>473.5149479351156</v>
+        <v>892.6683802523603</v>
       </c>
       <c r="CU4" t="n">
-        <v>472.3678063086063</v>
+        <v>892.3169514810401</v>
       </c>
       <c r="CV4" t="n">
-        <v>440.5998686011429</v>
+        <v>892.5377157651423</v>
       </c>
       <c r="CW4" t="n">
-        <v>468.4927220641788</v>
+        <v>995.2311002583843</v>
       </c>
     </row>
     <row r="5">
@@ -1638,304 +1638,304 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>447.9323216346033</v>
+        <v>1027.343936206536</v>
       </c>
       <c r="C5" t="n">
-        <v>481.2029200620591</v>
+        <v>1034.116321099957</v>
       </c>
       <c r="D5" t="n">
-        <v>495.341682135705</v>
+        <v>1041.065112435032</v>
       </c>
       <c r="E5" t="n">
-        <v>493.3116352945346</v>
+        <v>1041.671904073432</v>
       </c>
       <c r="F5" t="n">
-        <v>509.8228039020467</v>
+        <v>1037.29580769522</v>
       </c>
       <c r="G5" t="n">
-        <v>492.8398027523702</v>
+        <v>1041.967357183936</v>
       </c>
       <c r="H5" t="n">
-        <v>492.5389178048484</v>
+        <v>1046.417799665617</v>
       </c>
       <c r="I5" t="n">
-        <v>505.3427774656331</v>
+        <v>1040.91030622335</v>
       </c>
       <c r="J5" t="n">
-        <v>500.2602588189607</v>
+        <v>1043.028172437884</v>
       </c>
       <c r="K5" t="n">
-        <v>502.5765111329859</v>
+        <v>1041.070217982987</v>
       </c>
       <c r="L5" t="n">
-        <v>501.9256239066611</v>
+        <v>1033.306448213499</v>
       </c>
       <c r="M5" t="n">
-        <v>493.9963849711586</v>
+        <v>1037.238602067875</v>
       </c>
       <c r="N5" t="n">
-        <v>507.177147527815</v>
+        <v>1043.229365646232</v>
       </c>
       <c r="O5" t="n">
-        <v>499.8330746778271</v>
+        <v>1041.505291053368</v>
       </c>
       <c r="P5" t="n">
-        <v>494.4297923002397</v>
+        <v>1042.738599925124</v>
       </c>
       <c r="Q5" t="n">
-        <v>504.0619404445785</v>
+        <v>1015.457441892338</v>
       </c>
       <c r="R5" t="n">
-        <v>504.8887750880898</v>
+        <v>1041.710310523521</v>
       </c>
       <c r="S5" t="n">
-        <v>499.7845302963906</v>
+        <v>1044.369966634909</v>
       </c>
       <c r="T5" t="n">
-        <v>462.2653502276574</v>
+        <v>1018.455738407449</v>
       </c>
       <c r="U5" t="n">
-        <v>457.6599733542328</v>
+        <v>1014.622814337023</v>
       </c>
       <c r="V5" t="n">
-        <v>507.949429748987</v>
+        <v>1017.569141583906</v>
       </c>
       <c r="W5" t="n">
-        <v>439.2240281363531</v>
+        <v>1042.286114988325</v>
       </c>
       <c r="X5" t="n">
-        <v>495.1863721473616</v>
+        <v>962.7198164025173</v>
       </c>
       <c r="Y5" t="n">
-        <v>465.5053933786109</v>
+        <v>1041.166341368316</v>
       </c>
       <c r="Z5" t="n">
-        <v>441.1267342773996</v>
+        <v>957.7896855996969</v>
       </c>
       <c r="AA5" t="n">
-        <v>465.1704196713624</v>
+        <v>1018.521488787138</v>
       </c>
       <c r="AB5" t="n">
-        <v>442.4569362538006</v>
+        <v>1020.375833401785</v>
       </c>
       <c r="AC5" t="n">
-        <v>499.5255322930675</v>
+        <v>960.3106534740357</v>
       </c>
       <c r="AD5" t="n">
-        <v>454.8040214438476</v>
+        <v>997.2122567263352</v>
       </c>
       <c r="AE5" t="n">
-        <v>460.3088863663555</v>
+        <v>913.2955360925804</v>
       </c>
       <c r="AF5" t="n">
-        <v>443.3680388564262</v>
+        <v>996.9461694551086</v>
       </c>
       <c r="AG5" t="n">
-        <v>504.6416072041148</v>
+        <v>895.4584940935777</v>
       </c>
       <c r="AH5" t="n">
-        <v>436.2829803895678</v>
+        <v>934.7064058997814</v>
       </c>
       <c r="AI5" t="n">
-        <v>441.0232196447922</v>
+        <v>999.3953222232491</v>
       </c>
       <c r="AJ5" t="n">
-        <v>464.5753792332392</v>
+        <v>895.2913640863659</v>
       </c>
       <c r="AK5" t="n">
-        <v>444.2141586762804</v>
+        <v>997.2780672907604</v>
       </c>
       <c r="AL5" t="n">
-        <v>501.1425007125587</v>
+        <v>892.8190987978287</v>
       </c>
       <c r="AM5" t="n">
-        <v>488.3150309082283</v>
+        <v>895.2661148450832</v>
       </c>
       <c r="AN5" t="n">
-        <v>460.8995080488254</v>
+        <v>939.3101719171455</v>
       </c>
       <c r="AO5" t="n">
-        <v>487.7178291728023</v>
+        <v>912.6901369491998</v>
       </c>
       <c r="AP5" t="n">
-        <v>441.0879846890264</v>
+        <v>935.1897205839532</v>
       </c>
       <c r="AQ5" t="n">
-        <v>429.7611447670484</v>
+        <v>939.5346019305838</v>
       </c>
       <c r="AR5" t="n">
-        <v>461.1304240528516</v>
+        <v>894.8016075180403</v>
       </c>
       <c r="AS5" t="n">
-        <v>475.1128021019142</v>
+        <v>994.829410609122</v>
       </c>
       <c r="AT5" t="n">
-        <v>490.7088166967895</v>
+        <v>939.3646267082364</v>
       </c>
       <c r="AU5" t="n">
-        <v>493.7911485768386</v>
+        <v>892.2671116537409</v>
       </c>
       <c r="AV5" t="n">
-        <v>432.8826513080284</v>
+        <v>892.7345565870826</v>
       </c>
       <c r="AW5" t="n">
-        <v>446.1578394676841</v>
+        <v>894.9448535696094</v>
       </c>
       <c r="AX5" t="n">
-        <v>442.3384589694844</v>
+        <v>895.1367749272658</v>
       </c>
       <c r="AY5" t="n">
-        <v>441.3824353067779</v>
+        <v>937.6968109028206</v>
       </c>
       <c r="AZ5" t="n">
-        <v>485.6442524612379</v>
+        <v>897.1721777866421</v>
       </c>
       <c r="BA5" t="n">
-        <v>427.657381266307</v>
+        <v>892.2949265231048</v>
       </c>
       <c r="BB5" t="n">
-        <v>434.7556088432501</v>
+        <v>995.5012038759749</v>
       </c>
       <c r="BC5" t="n">
-        <v>439.0587726497553</v>
+        <v>993.3208953345268</v>
       </c>
       <c r="BD5" t="n">
-        <v>223.8304529332202</v>
+        <v>994.3423045214855</v>
       </c>
       <c r="BE5" t="n">
-        <v>349.0119341623152</v>
+        <v>934.379425836767</v>
       </c>
       <c r="BF5" t="n">
-        <v>419.0886293587333</v>
+        <v>894.9123322864891</v>
       </c>
       <c r="BG5" t="n">
-        <v>485.4694442072652</v>
+        <v>992.6084912824263</v>
       </c>
       <c r="BH5" t="n">
-        <v>462.5318392682839</v>
+        <v>891.8287096638351</v>
       </c>
       <c r="BI5" t="n">
-        <v>460.9477432221711</v>
+        <v>934.6510863127899</v>
       </c>
       <c r="BJ5" t="n">
-        <v>468.2363340021099</v>
+        <v>934.6385530589694</v>
       </c>
       <c r="BK5" t="n">
-        <v>427.4848673119407</v>
+        <v>892.4435649715781</v>
       </c>
       <c r="BL5" t="n">
-        <v>413.4481482096893</v>
+        <v>892.5598581092461</v>
       </c>
       <c r="BM5" t="n">
-        <v>414.2988794232926</v>
+        <v>939.3983905639727</v>
       </c>
       <c r="BN5" t="n">
-        <v>431.3522284465912</v>
+        <v>937.2282053044155</v>
       </c>
       <c r="BO5" t="n">
-        <v>401.2268227767149</v>
+        <v>892.6762677287392</v>
       </c>
       <c r="BP5" t="n">
-        <v>283.8694048099384</v>
+        <v>934.8105834689553</v>
       </c>
       <c r="BQ5" t="n">
-        <v>345.5570423793334</v>
+        <v>897.527342439325</v>
       </c>
       <c r="BR5" t="n">
-        <v>277.4561114389369</v>
+        <v>897.7364088316524</v>
       </c>
       <c r="BS5" t="n">
-        <v>288.7192702025337</v>
+        <v>892.5544933075234</v>
       </c>
       <c r="BT5" t="n">
-        <v>206.1549802800466</v>
+        <v>894.8686924199094</v>
       </c>
       <c r="BU5" t="n">
-        <v>481.5915152334688</v>
+        <v>892.0773893946209</v>
       </c>
       <c r="BV5" t="n">
-        <v>465.0091644684435</v>
+        <v>893.8254197831648</v>
       </c>
       <c r="BW5" t="n">
-        <v>493.4346433590889</v>
+        <v>892.5938738126672</v>
       </c>
       <c r="BX5" t="n">
-        <v>490.409162631619</v>
+        <v>894.9353908537872</v>
       </c>
       <c r="BY5" t="n">
-        <v>506.5252809628793</v>
+        <v>892.8321815982647</v>
       </c>
       <c r="BZ5" t="n">
-        <v>442.9923568073261</v>
+        <v>893.1934866249907</v>
       </c>
       <c r="CA5" t="n">
-        <v>465.0824892604251</v>
+        <v>893.0785680085592</v>
       </c>
       <c r="CB5" t="n">
-        <v>464.1273430115328</v>
+        <v>892.8432937471574</v>
       </c>
       <c r="CC5" t="n">
-        <v>434.8595291762122</v>
+        <v>894.7443422154108</v>
       </c>
       <c r="CD5" t="n">
-        <v>434.9473068886006</v>
+        <v>893.1477813312213</v>
       </c>
       <c r="CE5" t="n">
-        <v>431.8123790981648</v>
+        <v>897.8200617984861</v>
       </c>
       <c r="CF5" t="n">
-        <v>432.0583810769822</v>
+        <v>897.7955425287319</v>
       </c>
       <c r="CG5" t="n">
-        <v>426.0967692530152</v>
+        <v>892.4772391311083</v>
       </c>
       <c r="CH5" t="n">
-        <v>441.3026571810516</v>
+        <v>892.402304809945</v>
       </c>
       <c r="CI5" t="n">
-        <v>314.4284248891569</v>
+        <v>892.3831453865008</v>
       </c>
       <c r="CJ5" t="n">
-        <v>366.3366828190495</v>
+        <v>895.2196820936867</v>
       </c>
       <c r="CK5" t="n">
-        <v>266.1823814327531</v>
+        <v>894.8132263529317</v>
       </c>
       <c r="CL5" t="n">
-        <v>299.1791347557958</v>
+        <v>889.6183804548582</v>
       </c>
       <c r="CM5" t="n">
-        <v>364.1389972489948</v>
+        <v>892.4626766363599</v>
       </c>
       <c r="CN5" t="n">
-        <v>255.6085591200063</v>
+        <v>892.4580999670659</v>
       </c>
       <c r="CO5" t="n">
-        <v>271.8148867840877</v>
+        <v>894.8987351948419</v>
       </c>
       <c r="CP5" t="n">
-        <v>268.0536426478473</v>
+        <v>892.6360135328481</v>
       </c>
       <c r="CQ5" t="n">
-        <v>269.3240313901481</v>
+        <v>894.9289504214692</v>
       </c>
       <c r="CR5" t="n">
-        <v>269.0270393139573</v>
+        <v>892.4334152161164</v>
       </c>
       <c r="CS5" t="n">
-        <v>292.1370965146202</v>
+        <v>892.5463307827588</v>
       </c>
       <c r="CT5" t="n">
-        <v>473.5149479351156</v>
+        <v>892.6683802523603</v>
       </c>
       <c r="CU5" t="n">
-        <v>472.3678063086063</v>
+        <v>892.3169514810401</v>
       </c>
       <c r="CV5" t="n">
-        <v>440.5998686011429</v>
+        <v>892.5377157651423</v>
       </c>
       <c r="CW5" t="n">
-        <v>456.5411777547151</v>
+        <v>995.2311002583843</v>
       </c>
     </row>
     <row r="6">
@@ -1943,304 +1943,304 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>448.5295791701986</v>
+        <v>1026.26270244142</v>
       </c>
       <c r="C6" t="n">
-        <v>481.2029200620591</v>
+        <v>1034.116321099957</v>
       </c>
       <c r="D6" t="n">
-        <v>495.341682135705</v>
+        <v>1041.065112435032</v>
       </c>
       <c r="E6" t="n">
-        <v>493.3116352945346</v>
+        <v>1041.671904073432</v>
       </c>
       <c r="F6" t="n">
-        <v>507.7587577400673</v>
+        <v>1037.29580769522</v>
       </c>
       <c r="G6" t="n">
-        <v>492.8398027523702</v>
+        <v>1041.967357183936</v>
       </c>
       <c r="H6" t="n">
-        <v>492.5389178048484</v>
+        <v>1046.417799665617</v>
       </c>
       <c r="I6" t="n">
-        <v>505.3427774656331</v>
+        <v>1040.91030622335</v>
       </c>
       <c r="J6" t="n">
-        <v>500.2602588189607</v>
+        <v>1040.986266009831</v>
       </c>
       <c r="K6" t="n">
-        <v>502.5765111329859</v>
+        <v>1041.070217982987</v>
       </c>
       <c r="L6" t="n">
-        <v>501.9256239066611</v>
+        <v>1033.306448213499</v>
       </c>
       <c r="M6" t="n">
-        <v>493.9963849711586</v>
+        <v>1046.980329543537</v>
       </c>
       <c r="N6" t="n">
-        <v>507.177147527815</v>
+        <v>1043.229365646232</v>
       </c>
       <c r="O6" t="n">
-        <v>499.8330746778271</v>
+        <v>1017.311692666036</v>
       </c>
       <c r="P6" t="n">
-        <v>494.4297923002397</v>
+        <v>1018.386311411347</v>
       </c>
       <c r="Q6" t="n">
-        <v>504.0619404445785</v>
+        <v>995.3060825979574</v>
       </c>
       <c r="R6" t="n">
-        <v>504.8887750880898</v>
+        <v>960.3798494776071</v>
       </c>
       <c r="S6" t="n">
-        <v>461.7132812761711</v>
+        <v>1019.98090755049</v>
       </c>
       <c r="T6" t="n">
-        <v>462.2653502276574</v>
+        <v>998.2065031270915</v>
       </c>
       <c r="U6" t="n">
-        <v>457.6599733542328</v>
+        <v>997.247082108526</v>
       </c>
       <c r="V6" t="n">
-        <v>507.949429748987</v>
+        <v>1017.569141583906</v>
       </c>
       <c r="W6" t="n">
-        <v>439.2240281363531</v>
+        <v>1044.694983971076</v>
       </c>
       <c r="X6" t="n">
-        <v>456.4655528403006</v>
+        <v>962.7198164025173</v>
       </c>
       <c r="Y6" t="n">
-        <v>465.5053933786109</v>
+        <v>1020.039085412323</v>
       </c>
       <c r="Z6" t="n">
-        <v>441.1267342773996</v>
+        <v>915.9433321959357</v>
       </c>
       <c r="AA6" t="n">
-        <v>465.1704196713624</v>
+        <v>998.2722535067805</v>
       </c>
       <c r="AB6" t="n">
-        <v>429.4105844142658</v>
+        <v>1020.375833401785</v>
       </c>
       <c r="AC6" t="n">
-        <v>499.5255322930675</v>
+        <v>939.8889355223868</v>
       </c>
       <c r="AD6" t="n">
-        <v>432.3210488892497</v>
+        <v>937.3253499135546</v>
       </c>
       <c r="AE6" t="n">
-        <v>441.2265558243092</v>
+        <v>913.2955360925804</v>
       </c>
       <c r="AF6" t="n">
-        <v>443.3680388564262</v>
+        <v>892.909112835169</v>
       </c>
       <c r="AG6" t="n">
-        <v>504.6416072041148</v>
+        <v>895.4584940935777</v>
       </c>
       <c r="AH6" t="n">
-        <v>436.2829803895678</v>
+        <v>934.7064058997814</v>
       </c>
       <c r="AI6" t="n">
-        <v>441.0232196447922</v>
+        <v>999.3953222232491</v>
       </c>
       <c r="AJ6" t="n">
-        <v>419.3005442700143</v>
+        <v>892.7856544577742</v>
       </c>
       <c r="AK6" t="n">
-        <v>438.3795043324235</v>
+        <v>936.8032849132433</v>
       </c>
       <c r="AL6" t="n">
-        <v>486.493669552844</v>
+        <v>892.8190987978287</v>
       </c>
       <c r="AM6" t="n">
-        <v>482.5724423845231</v>
+        <v>892.7661148450832</v>
       </c>
       <c r="AN6" t="n">
-        <v>460.8995080488254</v>
+        <v>939.3101719171455</v>
       </c>
       <c r="AO6" t="n">
-        <v>313.9185985301339</v>
+        <v>892.9901905970357</v>
       </c>
       <c r="AP6" t="n">
-        <v>441.0879846890264</v>
+        <v>935.1897205839532</v>
       </c>
       <c r="AQ6" t="n">
-        <v>429.7611447670484</v>
+        <v>939.5346019305838</v>
       </c>
       <c r="AR6" t="n">
-        <v>444.292642164779</v>
+        <v>894.8016075180403</v>
       </c>
       <c r="AS6" t="n">
-        <v>470.9405202070442</v>
+        <v>995.6058038113721</v>
       </c>
       <c r="AT6" t="n">
-        <v>374.9443850405697</v>
+        <v>939.3646267082364</v>
       </c>
       <c r="AU6" t="n">
-        <v>378.2482380245446</v>
+        <v>892.2671116537409</v>
       </c>
       <c r="AV6" t="n">
-        <v>318.5856001748792</v>
+        <v>892.7345565870826</v>
       </c>
       <c r="AW6" t="n">
-        <v>446.1578394676841</v>
+        <v>894.9448535696094</v>
       </c>
       <c r="AX6" t="n">
-        <v>435.3119334288091</v>
+        <v>892.5242965536281</v>
       </c>
       <c r="AY6" t="n">
-        <v>423.1544801851129</v>
+        <v>890.5008925536831</v>
       </c>
       <c r="AZ6" t="n">
-        <v>483.8893254915527</v>
+        <v>893.9313442931146</v>
       </c>
       <c r="BA6" t="n">
-        <v>427.657381266307</v>
+        <v>892.2949265231048</v>
       </c>
       <c r="BB6" t="n">
-        <v>422.0828150449359</v>
+        <v>937.2585672027141</v>
       </c>
       <c r="BC6" t="n">
-        <v>439.0587726497553</v>
+        <v>995.8729082052847</v>
       </c>
       <c r="BD6" t="n">
-        <v>219.7698205616682</v>
+        <v>937.1669945926666</v>
       </c>
       <c r="BE6" t="n">
-        <v>256.1276969336941</v>
+        <v>892.5330724330058</v>
       </c>
       <c r="BF6" t="n">
-        <v>419.0886293587333</v>
+        <v>894.9123322864891</v>
       </c>
       <c r="BG6" t="n">
-        <v>485.4694442072652</v>
+        <v>931.9651185015288</v>
       </c>
       <c r="BH6" t="n">
-        <v>462.5318392682839</v>
+        <v>891.8287096638351</v>
       </c>
       <c r="BI6" t="n">
-        <v>460.9477432221711</v>
+        <v>934.6510863127899</v>
       </c>
       <c r="BJ6" t="n">
-        <v>451.3240867012167</v>
+        <v>934.6385530589694</v>
       </c>
       <c r="BK6" t="n">
-        <v>415.6833049072965</v>
+        <v>892.4435649715781</v>
       </c>
       <c r="BL6" t="n">
-        <v>413.4481482096893</v>
+        <v>892.5598581092461</v>
       </c>
       <c r="BM6" t="n">
-        <v>292.3228622633544</v>
+        <v>936.8969622839702</v>
       </c>
       <c r="BN6" t="n">
-        <v>431.3522284465912</v>
+        <v>937.2282053044155</v>
       </c>
       <c r="BO6" t="n">
-        <v>401.2268227767149</v>
+        <v>892.6762677287392</v>
       </c>
       <c r="BP6" t="n">
-        <v>283.8694048099384</v>
+        <v>934.8105834689553</v>
       </c>
       <c r="BQ6" t="n">
-        <v>247.1176545040834</v>
+        <v>894.921791163861</v>
       </c>
       <c r="BR6" t="n">
-        <v>277.4561114389369</v>
+        <v>897.7364088316524</v>
       </c>
       <c r="BS6" t="n">
-        <v>288.7192702025337</v>
+        <v>892.5544933075234</v>
       </c>
       <c r="BT6" t="n">
-        <v>206.1549802800466</v>
+        <v>894.8686924199094</v>
       </c>
       <c r="BU6" t="n">
-        <v>465.888996514161</v>
+        <v>892.9773893946209</v>
       </c>
       <c r="BV6" t="n">
-        <v>461.0847355675454</v>
+        <v>894.7254197831647</v>
       </c>
       <c r="BW6" t="n">
-        <v>475.8659627482458</v>
+        <v>892.5938738126672</v>
       </c>
       <c r="BX6" t="n">
-        <v>490.409162631619</v>
+        <v>894.9353908537872</v>
       </c>
       <c r="BY6" t="n">
-        <v>486.4328652643397</v>
+        <v>892.8321815982647</v>
       </c>
       <c r="BZ6" t="n">
-        <v>442.9923568073261</v>
+        <v>893.1934866249907</v>
       </c>
       <c r="CA6" t="n">
-        <v>465.0824892604251</v>
+        <v>893.0785680085592</v>
       </c>
       <c r="CB6" t="n">
-        <v>464.1273430115328</v>
+        <v>892.8432937471574</v>
       </c>
       <c r="CC6" t="n">
-        <v>434.8595291762122</v>
+        <v>894.7443422154108</v>
       </c>
       <c r="CD6" t="n">
-        <v>318.4061970588904</v>
+        <v>893.1477813312213</v>
       </c>
       <c r="CE6" t="n">
-        <v>414.1098688032404</v>
+        <v>897.8200617984861</v>
       </c>
       <c r="CF6" t="n">
-        <v>415.086667190989</v>
+        <v>897.7955425287319</v>
       </c>
       <c r="CG6" t="n">
-        <v>426.0967692530152</v>
+        <v>892.4772391311083</v>
       </c>
       <c r="CH6" t="n">
-        <v>326.1176215697475</v>
+        <v>892.402304809945</v>
       </c>
       <c r="CI6" t="n">
-        <v>314.4284248891569</v>
+        <v>892.3831453865008</v>
       </c>
       <c r="CJ6" t="n">
-        <v>366.3366828190495</v>
+        <v>895.2196820936867</v>
       </c>
       <c r="CK6" t="n">
-        <v>266.1823814327531</v>
+        <v>894.8132263529317</v>
       </c>
       <c r="CL6" t="n">
-        <v>299.1791347557958</v>
+        <v>889.6183804548582</v>
       </c>
       <c r="CM6" t="n">
-        <v>364.1389972489948</v>
+        <v>892.4626766363599</v>
       </c>
       <c r="CN6" t="n">
-        <v>255.6085591200063</v>
+        <v>892.4580999670659</v>
       </c>
       <c r="CO6" t="n">
-        <v>259.3107274823736</v>
+        <v>894.8987351948419</v>
       </c>
       <c r="CP6" t="n">
-        <v>268.0536426478473</v>
+        <v>892.6360135328481</v>
       </c>
       <c r="CQ6" t="n">
-        <v>257.099051563435</v>
+        <v>894.9289504214692</v>
       </c>
       <c r="CR6" t="n">
-        <v>269.0270393139573</v>
+        <v>892.4334152161164</v>
       </c>
       <c r="CS6" t="n">
-        <v>268.2170242835853</v>
+        <v>892.5463307827588</v>
       </c>
       <c r="CT6" t="n">
-        <v>461.3905431867089</v>
+        <v>892.6683802523603</v>
       </c>
       <c r="CU6" t="n">
-        <v>472.3678063086063</v>
+        <v>892.3169514810401</v>
       </c>
       <c r="CV6" t="n">
-        <v>440.5998686011429</v>
+        <v>892.5377157651423</v>
       </c>
       <c r="CW6" t="n">
-        <v>456.5411777547151</v>
+        <v>995.2311002583843</v>
       </c>
     </row>
     <row r="7">
@@ -2248,304 +2248,304 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>481.3740692313619</v>
+        <v>1026.26270244142</v>
       </c>
       <c r="C7" t="n">
-        <v>481.2029200620591</v>
+        <v>1034.116321099957</v>
       </c>
       <c r="D7" t="n">
-        <v>495.341682135705</v>
+        <v>1041.065112435032</v>
       </c>
       <c r="E7" t="n">
-        <v>493.3116352945346</v>
+        <v>1041.671904073432</v>
       </c>
       <c r="F7" t="n">
-        <v>492.877845036049</v>
+        <v>1042.254136376345</v>
       </c>
       <c r="G7" t="n">
-        <v>492.8398027523702</v>
+        <v>1041.967357183936</v>
       </c>
       <c r="H7" t="n">
-        <v>492.5389178048484</v>
+        <v>1046.417799665617</v>
       </c>
       <c r="I7" t="n">
-        <v>505.3427774656331</v>
+        <v>1040.91030622335</v>
       </c>
       <c r="J7" t="n">
-        <v>500.2602588189607</v>
+        <v>1040.986266009831</v>
       </c>
       <c r="K7" t="n">
-        <v>502.5765111329859</v>
+        <v>1041.070217982987</v>
       </c>
       <c r="L7" t="n">
-        <v>501.9256239066611</v>
+        <v>1033.306448213499</v>
       </c>
       <c r="M7" t="n">
-        <v>465.9705344237586</v>
+        <v>1022.498325284937</v>
       </c>
       <c r="N7" t="n">
-        <v>507.177147527815</v>
+        <v>1043.229365646232</v>
       </c>
       <c r="O7" t="n">
-        <v>468.1588382969989</v>
+        <v>1017.311692666036</v>
       </c>
       <c r="P7" t="n">
-        <v>494.4297923002397</v>
+        <v>1018.386311411347</v>
       </c>
       <c r="Q7" t="n">
-        <v>504.0619404445785</v>
+        <v>997.5541652219642</v>
       </c>
       <c r="R7" t="n">
-        <v>504.8887750880898</v>
+        <v>960.3798494776071</v>
       </c>
       <c r="S7" t="n">
-        <v>461.7132812761711</v>
+        <v>1019.98090755049</v>
       </c>
       <c r="T7" t="n">
-        <v>462.2653502276574</v>
+        <v>998.2065031270915</v>
       </c>
       <c r="U7" t="n">
-        <v>438.4698148605509</v>
+        <v>997.247082108526</v>
       </c>
       <c r="V7" t="n">
-        <v>507.949429748987</v>
+        <v>955.1606248057948</v>
       </c>
       <c r="W7" t="n">
-        <v>439.2240281363531</v>
+        <v>1020.303505679365</v>
       </c>
       <c r="X7" t="n">
-        <v>456.4655528403006</v>
+        <v>942.2475086550952</v>
       </c>
       <c r="Y7" t="n">
-        <v>465.5053933786109</v>
+        <v>999.9239249819593</v>
       </c>
       <c r="Z7" t="n">
-        <v>441.1267342773996</v>
+        <v>915.9433321959357</v>
       </c>
       <c r="AA7" t="n">
-        <v>465.1704196713624</v>
+        <v>998.2722535067805</v>
       </c>
       <c r="AB7" t="n">
-        <v>429.4105844142658</v>
+        <v>1020.375833401785</v>
       </c>
       <c r="AC7" t="n">
-        <v>499.5255322930675</v>
+        <v>939.8889355223868</v>
       </c>
       <c r="AD7" t="n">
-        <v>432.3210488892497</v>
+        <v>895.4836396972769</v>
       </c>
       <c r="AE7" t="n">
-        <v>428.0498143087141</v>
+        <v>916.0118603974872</v>
       </c>
       <c r="AF7" t="n">
-        <v>443.3680388564262</v>
+        <v>892.909112835169</v>
       </c>
       <c r="AG7" t="n">
-        <v>504.6416072041148</v>
+        <v>895.4584940935777</v>
       </c>
       <c r="AH7" t="n">
-        <v>436.2829803895678</v>
+        <v>934.7064058997814</v>
       </c>
       <c r="AI7" t="n">
-        <v>305.6771447447913</v>
+        <v>999.3953222232491</v>
       </c>
       <c r="AJ7" t="n">
-        <v>419.3005442700143</v>
+        <v>892.7856544577742</v>
       </c>
       <c r="AK7" t="n">
-        <v>425.0512106447579</v>
+        <v>892.3817041393424</v>
       </c>
       <c r="AL7" t="n">
-        <v>482.714428239974</v>
+        <v>892.8190987978287</v>
       </c>
       <c r="AM7" t="n">
-        <v>482.5724423845231</v>
+        <v>892.7661148450832</v>
       </c>
       <c r="AN7" t="n">
-        <v>455.2144500834821</v>
+        <v>892.5745616414624</v>
       </c>
       <c r="AO7" t="n">
-        <v>301.7784497841657</v>
+        <v>892.9901905970357</v>
       </c>
       <c r="AP7" t="n">
-        <v>427.9766417338007</v>
+        <v>935.1897205839532</v>
       </c>
       <c r="AQ7" t="n">
-        <v>412.2364878368156</v>
+        <v>937.0331736505814</v>
       </c>
       <c r="AR7" t="n">
-        <v>412.8836930517267</v>
+        <v>894.8016075180403</v>
       </c>
       <c r="AS7" t="n">
-        <v>459.1342717321785</v>
+        <v>934.4726754008419</v>
       </c>
       <c r="AT7" t="n">
-        <v>374.9443850405697</v>
+        <v>939.3646267082364</v>
       </c>
       <c r="AU7" t="n">
-        <v>355.7220823674892</v>
+        <v>892.2671116537409</v>
       </c>
       <c r="AV7" t="n">
-        <v>318.5856001748792</v>
+        <v>892.7345565870826</v>
       </c>
       <c r="AW7" t="n">
-        <v>423.360384649128</v>
+        <v>892.4448535696094</v>
       </c>
       <c r="AX7" t="n">
-        <v>418.9694278428217</v>
+        <v>892.5242965536281</v>
       </c>
       <c r="AY7" t="n">
-        <v>411.6280082157194</v>
+        <v>892.6874795834207</v>
       </c>
       <c r="AZ7" t="n">
-        <v>466.5034904723975</v>
+        <v>894.5707891655684</v>
       </c>
       <c r="BA7" t="n">
-        <v>427.657381266307</v>
+        <v>892.2949265231048</v>
       </c>
       <c r="BB7" t="n">
-        <v>422.0828150449359</v>
+        <v>892.4772391311083</v>
       </c>
       <c r="BC7" t="n">
-        <v>303.260883130623</v>
+        <v>892.822776962554</v>
       </c>
       <c r="BD7" t="n">
-        <v>206.5930790460729</v>
+        <v>937.1669945926666</v>
       </c>
       <c r="BE7" t="n">
-        <v>214.4484392404428</v>
+        <v>892.5330724330058</v>
       </c>
       <c r="BF7" t="n">
-        <v>419.0886293587333</v>
+        <v>894.9123322864891</v>
       </c>
       <c r="BG7" t="n">
-        <v>473.076553226698</v>
+        <v>892.599248767728</v>
       </c>
       <c r="BH7" t="n">
-        <v>462.5318392682839</v>
+        <v>891.8287096638351</v>
       </c>
       <c r="BI7" t="n">
-        <v>460.9477432221711</v>
+        <v>934.6510863127899</v>
       </c>
       <c r="BJ7" t="n">
-        <v>440.1122072389882</v>
+        <v>892.4995915508385</v>
       </c>
       <c r="BK7" t="n">
-        <v>415.6833049072965</v>
+        <v>892.4435649715781</v>
       </c>
       <c r="BL7" t="n">
-        <v>413.4481482096893</v>
+        <v>892.5598581092461</v>
       </c>
       <c r="BM7" t="n">
-        <v>292.3228622633544</v>
+        <v>892.5745616414624</v>
       </c>
       <c r="BN7" t="n">
-        <v>411.0644385190295</v>
+        <v>937.2282053044155</v>
       </c>
       <c r="BO7" t="n">
-        <v>401.2268227767149</v>
+        <v>892.6762677287392</v>
       </c>
       <c r="BP7" t="n">
-        <v>283.8694048099384</v>
+        <v>892.5410791963155</v>
       </c>
       <c r="BQ7" t="n">
-        <v>247.1176545040834</v>
+        <v>894.921791163861</v>
       </c>
       <c r="BR7" t="n">
-        <v>277.4561114389369</v>
+        <v>897.7364088316524</v>
       </c>
       <c r="BS7" t="n">
-        <v>277.331271978446</v>
+        <v>892.5544933075234</v>
       </c>
       <c r="BT7" t="n">
-        <v>206.1549802800466</v>
+        <v>894.8686924199094</v>
       </c>
       <c r="BU7" t="n">
-        <v>465.888996514161</v>
+        <v>892.9773893946209</v>
       </c>
       <c r="BV7" t="n">
-        <v>461.0847355675454</v>
+        <v>894.7254197831647</v>
       </c>
       <c r="BW7" t="n">
-        <v>463.884726289418</v>
+        <v>892.5938738126672</v>
       </c>
       <c r="BX7" t="n">
-        <v>490.409162631619</v>
+        <v>894.9353908537872</v>
       </c>
       <c r="BY7" t="n">
-        <v>486.4328652643397</v>
+        <v>892.8321815982647</v>
       </c>
       <c r="BZ7" t="n">
-        <v>442.9923568073261</v>
+        <v>893.1934866249907</v>
       </c>
       <c r="CA7" t="n">
-        <v>453.3627211807783</v>
+        <v>893.0785680085592</v>
       </c>
       <c r="CB7" t="n">
-        <v>464.1273430115328</v>
+        <v>892.8432937471574</v>
       </c>
       <c r="CC7" t="n">
-        <v>417.7851688832446</v>
+        <v>894.7443422154108</v>
       </c>
       <c r="CD7" t="n">
-        <v>318.4061970588904</v>
+        <v>893.1477813312213</v>
       </c>
       <c r="CE7" t="n">
-        <v>414.1098688032404</v>
+        <v>897.8200617984861</v>
       </c>
       <c r="CF7" t="n">
-        <v>279.1007420380499</v>
+        <v>897.7955425287319</v>
       </c>
       <c r="CG7" t="n">
-        <v>426.0967692530152</v>
+        <v>892.4772391311083</v>
       </c>
       <c r="CH7" t="n">
-        <v>293.7605117452528</v>
+        <v>892.402304809945</v>
       </c>
       <c r="CI7" t="n">
-        <v>314.4284248891569</v>
+        <v>892.3831453865008</v>
       </c>
       <c r="CJ7" t="n">
-        <v>346.0488928914878</v>
+        <v>895.2196820936867</v>
       </c>
       <c r="CK7" t="n">
-        <v>266.1823814327531</v>
+        <v>894.8132263529317</v>
       </c>
       <c r="CL7" t="n">
-        <v>299.1791347557958</v>
+        <v>889.6183804548582</v>
       </c>
       <c r="CM7" t="n">
-        <v>247.0114247510222</v>
+        <v>892.4626766363599</v>
       </c>
       <c r="CN7" t="n">
-        <v>255.6085591200063</v>
+        <v>892.4580999670659</v>
       </c>
       <c r="CO7" t="n">
-        <v>247.2046220349114</v>
+        <v>894.8987351948419</v>
       </c>
       <c r="CP7" t="n">
-        <v>254.8769011322521</v>
+        <v>892.6360135328481</v>
       </c>
       <c r="CQ7" t="n">
-        <v>257.099051563435</v>
+        <v>894.9289504214692</v>
       </c>
       <c r="CR7" t="n">
-        <v>269.0270393139573</v>
+        <v>892.4334152161164</v>
       </c>
       <c r="CS7" t="n">
-        <v>256.076875537617</v>
+        <v>892.5463307827588</v>
       </c>
       <c r="CT7" t="n">
-        <v>461.3905431867089</v>
+        <v>892.6683802523603</v>
       </c>
       <c r="CU7" t="n">
-        <v>472.3678063086063</v>
+        <v>892.3169514810401</v>
       </c>
       <c r="CV7" t="n">
-        <v>427.5641997535248</v>
+        <v>892.5377157651423</v>
       </c>
       <c r="CW7" t="n">
-        <v>456.5411777547151</v>
+        <v>995.2311002583843</v>
       </c>
     </row>
     <row r="8">
@@ -2553,304 +2553,304 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>481.3740692313619</v>
+        <v>1032.544681594848</v>
       </c>
       <c r="C8" t="n">
-        <v>481.2029200620591</v>
+        <v>1034.116321099957</v>
       </c>
       <c r="D8" t="n">
-        <v>495.341682135705</v>
+        <v>1041.065112435032</v>
       </c>
       <c r="E8" t="n">
-        <v>493.3116352945346</v>
+        <v>1041.671904073432</v>
       </c>
       <c r="F8" t="n">
-        <v>492.877845036049</v>
+        <v>1042.254136376345</v>
       </c>
       <c r="G8" t="n">
-        <v>492.8398027523702</v>
+        <v>1041.967357183936</v>
       </c>
       <c r="H8" t="n">
-        <v>492.5389178048484</v>
+        <v>1046.417799665617</v>
       </c>
       <c r="I8" t="n">
-        <v>505.3427774656331</v>
+        <v>1040.91030622335</v>
       </c>
       <c r="J8" t="n">
-        <v>500.2602588189607</v>
+        <v>1016.674757948937</v>
       </c>
       <c r="K8" t="n">
-        <v>502.5765111329859</v>
+        <v>1041.070217982987</v>
       </c>
       <c r="L8" t="n">
-        <v>501.9256239066611</v>
+        <v>1043.458041707672</v>
       </c>
       <c r="M8" t="n">
-        <v>465.9705344237586</v>
+        <v>1022.498325284937</v>
       </c>
       <c r="N8" t="n">
-        <v>507.177147527815</v>
+        <v>1043.229365646232</v>
       </c>
       <c r="O8" t="n">
-        <v>468.1588382969989</v>
+        <v>1017.311692666036</v>
       </c>
       <c r="P8" t="n">
-        <v>494.4297923002397</v>
+        <v>1018.386311411347</v>
       </c>
       <c r="Q8" t="n">
-        <v>504.0619404445785</v>
+        <v>997.5541652219642</v>
       </c>
       <c r="R8" t="n">
-        <v>465.6334577419834</v>
+        <v>915.8943572850409</v>
       </c>
       <c r="S8" t="n">
-        <v>461.7132812761711</v>
+        <v>960.2039275360936</v>
       </c>
       <c r="T8" t="n">
-        <v>449.1540072724317</v>
+        <v>998.2065031270915</v>
       </c>
       <c r="U8" t="n">
-        <v>425.8097208189105</v>
+        <v>997.247082108526</v>
       </c>
       <c r="V8" t="n">
-        <v>507.949429748987</v>
+        <v>937.722955018794</v>
       </c>
       <c r="W8" t="n">
-        <v>433.6316082468132</v>
+        <v>1017.802077399363</v>
       </c>
       <c r="X8" t="n">
-        <v>438.0574576557971</v>
+        <v>939.6461200340215</v>
       </c>
       <c r="Y8" t="n">
-        <v>465.5053933786109</v>
+        <v>999.9239249819593</v>
       </c>
       <c r="Z8" t="n">
-        <v>441.1267342773996</v>
+        <v>895.5216142442869</v>
       </c>
       <c r="AA8" t="n">
-        <v>446.0880268856408</v>
+        <v>998.2722535067805</v>
       </c>
       <c r="AB8" t="n">
-        <v>412.1093342210127</v>
+        <v>997.2173084058586</v>
       </c>
       <c r="AC8" t="n">
-        <v>465.7919822197565</v>
+        <v>939.8889355223868</v>
       </c>
       <c r="AD8" t="n">
-        <v>420.1966441408431</v>
+        <v>895.4836396972769</v>
       </c>
       <c r="AE8" t="n">
-        <v>428.0498143087141</v>
+        <v>895.5395526500652</v>
       </c>
       <c r="AF8" t="n">
-        <v>317.1789481274897</v>
+        <v>893.0281756622647</v>
       </c>
       <c r="AG8" t="n">
-        <v>459.1571420137717</v>
+        <v>892.7530926308478</v>
       </c>
       <c r="AH8" t="n">
-        <v>418.6144675698577</v>
+        <v>934.7064058997814</v>
       </c>
       <c r="AI8" t="n">
-        <v>286.5905881096568</v>
+        <v>996.8938939432467</v>
       </c>
       <c r="AJ8" t="n">
-        <v>419.3005442700143</v>
+        <v>892.7856544577742</v>
       </c>
       <c r="AK8" t="n">
-        <v>425.0512106447579</v>
+        <v>892.3817041393424</v>
       </c>
       <c r="AL8" t="n">
-        <v>469.5626210614702</v>
+        <v>892.8190987978287</v>
       </c>
       <c r="AM8" t="n">
-        <v>469.4284507272858</v>
+        <v>892.7661148450832</v>
       </c>
       <c r="AN8" t="n">
-        <v>455.2144500834821</v>
+        <v>892.5745616414624</v>
       </c>
       <c r="AO8" t="n">
-        <v>301.7784497841657</v>
+        <v>892.9901905970357</v>
       </c>
       <c r="AP8" t="n">
-        <v>427.9766417338007</v>
+        <v>892.8971115149677</v>
       </c>
       <c r="AQ8" t="n">
-        <v>412.2364878368156</v>
+        <v>937.0331736505814</v>
       </c>
       <c r="AR8" t="n">
-        <v>412.8836930517267</v>
+        <v>894.8016075180403</v>
       </c>
       <c r="AS8" t="n">
-        <v>459.1342717321785</v>
+        <v>934.4726754008419</v>
       </c>
       <c r="AT8" t="n">
-        <v>339.7594961455185</v>
+        <v>894.6793660017645</v>
       </c>
       <c r="AU8" t="n">
-        <v>355.7220823674892</v>
+        <v>892.2671116537409</v>
       </c>
       <c r="AV8" t="n">
-        <v>208.1446848043815</v>
+        <v>892.7345565870826</v>
       </c>
       <c r="AW8" t="n">
-        <v>423.360384649128</v>
+        <v>892.4448535696094</v>
       </c>
       <c r="AX8" t="n">
-        <v>418.9694278428217</v>
+        <v>892.5242965536281</v>
       </c>
       <c r="AY8" t="n">
-        <v>411.6280082157194</v>
+        <v>892.6874795834207</v>
       </c>
       <c r="AZ8" t="n">
-        <v>466.5034904723975</v>
+        <v>894.5707891655684</v>
       </c>
       <c r="BA8" t="n">
-        <v>427.657381266307</v>
+        <v>892.2949265231048</v>
       </c>
       <c r="BB8" t="n">
-        <v>409.9732765328448</v>
+        <v>892.4772391311083</v>
       </c>
       <c r="BC8" t="n">
-        <v>291.2013080992523</v>
+        <v>892.822776962554</v>
       </c>
       <c r="BD8" t="n">
-        <v>206.5930790460729</v>
+        <v>892.6213032486985</v>
       </c>
       <c r="BE8" t="n">
-        <v>191.1903993361141</v>
+        <v>892.5330724330058</v>
       </c>
       <c r="BF8" t="n">
-        <v>407.6974026236598</v>
+        <v>894.9123322864891</v>
       </c>
       <c r="BG8" t="n">
-        <v>473.076553226698</v>
+        <v>892.599248767728</v>
       </c>
       <c r="BH8" t="n">
-        <v>458.4463206123353</v>
+        <v>892.728709663835</v>
       </c>
       <c r="BI8" t="n">
-        <v>460.9477432221711</v>
+        <v>934.6510863127899</v>
       </c>
       <c r="BJ8" t="n">
-        <v>418.3851308762002</v>
+        <v>892.4995915508385</v>
       </c>
       <c r="BK8" t="n">
-        <v>415.6833049072965</v>
+        <v>892.4435649715781</v>
       </c>
       <c r="BL8" t="n">
-        <v>413.4481482096893</v>
+        <v>892.5598581092461</v>
       </c>
       <c r="BM8" t="n">
-        <v>292.3228622633544</v>
+        <v>892.5745616414624</v>
       </c>
       <c r="BN8" t="n">
-        <v>405.602240750468</v>
+        <v>934.8223280312302</v>
       </c>
       <c r="BO8" t="n">
-        <v>401.2268227767149</v>
+        <v>892.6762677287392</v>
       </c>
       <c r="BP8" t="n">
-        <v>189.995172270223</v>
+        <v>892.5410791963155</v>
       </c>
       <c r="BQ8" t="n">
-        <v>247.1176545040834</v>
+        <v>894.921791163861</v>
       </c>
       <c r="BR8" t="n">
-        <v>277.4561114389369</v>
+        <v>897.7364088316524</v>
       </c>
       <c r="BS8" t="n">
-        <v>277.331271978446</v>
+        <v>892.5544933075234</v>
       </c>
       <c r="BT8" t="n">
-        <v>206.1549802800466</v>
+        <v>894.8686924199094</v>
       </c>
       <c r="BU8" t="n">
-        <v>465.888996514161</v>
+        <v>892.9773893946209</v>
       </c>
       <c r="BV8" t="n">
-        <v>461.0847355675454</v>
+        <v>894.7254197831647</v>
       </c>
       <c r="BW8" t="n">
-        <v>463.884726289418</v>
+        <v>892.5938738126672</v>
       </c>
       <c r="BX8" t="n">
-        <v>473.163272683469</v>
+        <v>894.9353908537872</v>
       </c>
       <c r="BY8" t="n">
-        <v>486.4328652643397</v>
+        <v>892.8321815982647</v>
       </c>
       <c r="BZ8" t="n">
-        <v>425.323843987616</v>
+        <v>893.1934866249907</v>
       </c>
       <c r="CA8" t="n">
-        <v>453.3627211807783</v>
+        <v>893.0785680085592</v>
       </c>
       <c r="CB8" t="n">
-        <v>464.1273430115328</v>
+        <v>892.8432937471574</v>
       </c>
       <c r="CC8" t="n">
-        <v>417.7851688832446</v>
+        <v>894.7443422154108</v>
       </c>
       <c r="CD8" t="n">
-        <v>318.4061970588904</v>
+        <v>893.1477813312213</v>
       </c>
       <c r="CE8" t="n">
-        <v>414.1098688032404</v>
+        <v>897.8200617984861</v>
       </c>
       <c r="CF8" t="n">
-        <v>279.1007420380499</v>
+        <v>892.9553018667732</v>
       </c>
       <c r="CG8" t="n">
-        <v>397.0691684080853</v>
+        <v>892.4772391311083</v>
       </c>
       <c r="CH8" t="n">
-        <v>199.7115112244688</v>
+        <v>892.402304809945</v>
       </c>
       <c r="CI8" t="n">
-        <v>301.5630813842581</v>
+        <v>892.3831453865008</v>
       </c>
       <c r="CJ8" t="n">
-        <v>299.4435201322285</v>
+        <v>895.2196820936867</v>
       </c>
       <c r="CK8" t="n">
-        <v>253.2175431558583</v>
+        <v>894.8132263529317</v>
       </c>
       <c r="CL8" t="n">
-        <v>287.0547300073891</v>
+        <v>894.5687133747485</v>
       </c>
       <c r="CM8" t="n">
-        <v>247.0114247510222</v>
+        <v>892.4626766363599</v>
       </c>
       <c r="CN8" t="n">
-        <v>243.5489840886357</v>
+        <v>892.4580999670659</v>
       </c>
       <c r="CO8" t="n">
-        <v>247.2046220349114</v>
+        <v>894.8987351948419</v>
       </c>
       <c r="CP8" t="n">
-        <v>254.8769011322521</v>
+        <v>648.4919334493185</v>
       </c>
       <c r="CQ8" t="n">
-        <v>257.099051563435</v>
+        <v>894.9289504214692</v>
       </c>
       <c r="CR8" t="n">
-        <v>256.5116379614213</v>
+        <v>892.4334152161164</v>
       </c>
       <c r="CS8" t="n">
-        <v>256.076875537617</v>
+        <v>892.5463307827588</v>
       </c>
       <c r="CT8" t="n">
-        <v>461.3905431867089</v>
+        <v>892.6683802523603</v>
       </c>
       <c r="CU8" t="n">
-        <v>472.3678063086063</v>
+        <v>892.3169514810401</v>
       </c>
       <c r="CV8" t="n">
-        <v>427.5641997535248</v>
+        <v>648.450772008442</v>
       </c>
       <c r="CW8" t="n">
-        <v>456.5411777547151</v>
+        <v>995.2311002583843</v>
       </c>
     </row>
     <row r="9">
@@ -2858,304 +2858,304 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>481.3740692313619</v>
+        <v>1032.544681594848</v>
       </c>
       <c r="C9" t="n">
-        <v>481.2029200620591</v>
+        <v>1034.116321099957</v>
       </c>
       <c r="D9" t="n">
-        <v>495.341682135705</v>
+        <v>1041.065112435032</v>
       </c>
       <c r="E9" t="n">
-        <v>493.3116352945346</v>
+        <v>1041.671904073432</v>
       </c>
       <c r="F9" t="n">
-        <v>492.877845036049</v>
+        <v>1042.254136376345</v>
       </c>
       <c r="G9" t="n">
-        <v>492.8398027523702</v>
+        <v>1041.967357183936</v>
       </c>
       <c r="H9" t="n">
-        <v>492.5389178048484</v>
+        <v>1022.192656039303</v>
       </c>
       <c r="I9" t="n">
-        <v>505.3427774656331</v>
+        <v>1040.91030622335</v>
       </c>
       <c r="J9" t="n">
-        <v>500.2602588189607</v>
+        <v>1016.674757948937</v>
       </c>
       <c r="K9" t="n">
-        <v>502.5765111329859</v>
+        <v>1041.070217982987</v>
       </c>
       <c r="L9" t="n">
-        <v>501.9256239066611</v>
+        <v>1043.458041707672</v>
       </c>
       <c r="M9" t="n">
-        <v>465.9705344237586</v>
+        <v>1022.498325284937</v>
       </c>
       <c r="N9" t="n">
-        <v>507.177147527815</v>
+        <v>1043.229365646232</v>
       </c>
       <c r="O9" t="n">
-        <v>468.1588382969989</v>
+        <v>1017.311692666036</v>
       </c>
       <c r="P9" t="n">
-        <v>494.4297923002397</v>
+        <v>1018.386311411347</v>
       </c>
       <c r="Q9" t="n">
-        <v>466.0023970401213</v>
+        <v>997.5541652219642</v>
       </c>
       <c r="R9" t="n">
-        <v>465.6334577419834</v>
+        <v>895.4220495376188</v>
       </c>
       <c r="S9" t="n">
-        <v>461.7132812761711</v>
+        <v>939.7822095844446</v>
       </c>
       <c r="T9" t="n">
-        <v>429.5996889913502</v>
+        <v>998.2065031270915</v>
       </c>
       <c r="U9" t="n">
-        <v>425.8097208189105</v>
+        <v>997.247082108526</v>
       </c>
       <c r="V9" t="n">
-        <v>507.949429748987</v>
+        <v>937.722955018794</v>
       </c>
       <c r="W9" t="n">
-        <v>421.1398698910883</v>
+        <v>997.2435524034363</v>
       </c>
       <c r="X9" t="n">
-        <v>438.0574576557971</v>
+        <v>939.6461200340215</v>
       </c>
       <c r="Y9" t="n">
-        <v>448.2107585527816</v>
+        <v>999.9239249819593</v>
       </c>
       <c r="Z9" t="n">
-        <v>441.1267342773996</v>
+        <v>895.5216142442869</v>
       </c>
       <c r="AA9" t="n">
-        <v>446.0880268856408</v>
+        <v>998.2722535067805</v>
       </c>
       <c r="AB9" t="n">
-        <v>412.1093342210127</v>
+        <v>934.7311681861223</v>
       </c>
       <c r="AC9" t="n">
-        <v>465.7919822197565</v>
+        <v>939.8889355223868</v>
       </c>
       <c r="AD9" t="n">
-        <v>414.6230226123399</v>
+        <v>893.0704300641016</v>
       </c>
       <c r="AE9" t="n">
-        <v>410.8873261957206</v>
+        <v>892.8382015454008</v>
       </c>
       <c r="AF9" t="n">
-        <v>297.0931116489433</v>
+        <v>893.0281756622647</v>
       </c>
       <c r="AG9" t="n">
-        <v>459.1571420137717</v>
+        <v>892.7530926308478</v>
       </c>
       <c r="AH9" t="n">
-        <v>418.6144675698577</v>
+        <v>934.7064058997814</v>
       </c>
       <c r="AI9" t="n">
-        <v>198.0702964792011</v>
+        <v>937.1398118448599</v>
       </c>
       <c r="AJ9" t="n">
-        <v>297.7061891395709</v>
+        <v>892.7856544577742</v>
       </c>
       <c r="AK9" t="n">
-        <v>425.0512106447579</v>
+        <v>892.3817041393424</v>
       </c>
       <c r="AL9" t="n">
-        <v>469.5626210614702</v>
+        <v>892.8190987978287</v>
       </c>
       <c r="AM9" t="n">
-        <v>469.4284507272858</v>
+        <v>892.7661148450832</v>
       </c>
       <c r="AN9" t="n">
-        <v>452.9942016458612</v>
+        <v>890.3745616414624</v>
       </c>
       <c r="AO9" t="n">
-        <v>299.5582013465448</v>
+        <v>890.7901905970357</v>
       </c>
       <c r="AP9" t="n">
-        <v>427.9766417338007</v>
+        <v>892.8971115149677</v>
       </c>
       <c r="AQ9" t="n">
-        <v>412.2364878368156</v>
+        <v>937.0331736505814</v>
       </c>
       <c r="AR9" t="n">
-        <v>410.6634446141057</v>
+        <v>892.6016075180403</v>
       </c>
       <c r="AS9" t="n">
-        <v>456.9140232945576</v>
+        <v>932.272675400842</v>
       </c>
       <c r="AT9" t="n">
-        <v>337.5392477078975</v>
+        <v>890.2860150104859</v>
       </c>
       <c r="AU9" t="n">
-        <v>324.1639828907005</v>
+        <v>890.0671116537409</v>
       </c>
       <c r="AV9" t="n">
-        <v>205.9244363667606</v>
+        <v>890.5345565870826</v>
       </c>
       <c r="AW9" t="n">
-        <v>421.140136211507</v>
+        <v>890.2448535696094</v>
       </c>
       <c r="AX9" t="n">
-        <v>416.7491794052008</v>
+        <v>890.3242965536281</v>
       </c>
       <c r="AY9" t="n">
-        <v>409.4077597780985</v>
+        <v>890.4874795834206</v>
       </c>
       <c r="AZ9" t="n">
-        <v>464.2832420347766</v>
+        <v>892.3707891655683</v>
       </c>
       <c r="BA9" t="n">
-        <v>425.4371328286861</v>
+        <v>890.0949265231047</v>
       </c>
       <c r="BB9" t="n">
-        <v>407.7530280952239</v>
+        <v>890.2772391311082</v>
       </c>
       <c r="BC9" t="n">
-        <v>194.4711208078839</v>
+        <v>890.6227769625541</v>
       </c>
       <c r="BD9" t="n">
-        <v>193.116709688683</v>
+        <v>890.4213032486985</v>
       </c>
       <c r="BE9" t="n">
-        <v>188.9701508984932</v>
+        <v>890.3330724330059</v>
       </c>
       <c r="BF9" t="n">
-        <v>267.0152401999704</v>
+        <v>892.7123322864891</v>
       </c>
       <c r="BG9" t="n">
-        <v>470.8563047890769</v>
+        <v>890.3992487677281</v>
       </c>
       <c r="BH9" t="n">
-        <v>456.2260721747144</v>
+        <v>890.5287096638351</v>
       </c>
       <c r="BI9" t="n">
-        <v>458.7274947845502</v>
+        <v>932.4510863127898</v>
       </c>
       <c r="BJ9" t="n">
-        <v>416.1648824385792</v>
+        <v>890.2995915508385</v>
       </c>
       <c r="BK9" t="n">
-        <v>413.4630564696756</v>
+        <v>890.2435649715781</v>
       </c>
       <c r="BL9" t="n">
-        <v>411.2278997720683</v>
+        <v>890.3598581092461</v>
       </c>
       <c r="BM9" t="n">
-        <v>290.1026138257334</v>
+        <v>890.3745616414624</v>
       </c>
       <c r="BN9" t="n">
-        <v>287.7560089300691</v>
+        <v>932.6223280312303</v>
       </c>
       <c r="BO9" t="n">
-        <v>399.006574339094</v>
+        <v>890.4762677287392</v>
       </c>
       <c r="BP9" t="n">
-        <v>187.774923832602</v>
+        <v>890.3410791963155</v>
       </c>
       <c r="BQ9" t="n">
-        <v>244.8974060664625</v>
+        <v>892.7217911638611</v>
       </c>
       <c r="BR9" t="n">
-        <v>275.235863001316</v>
+        <v>895.5364088316525</v>
       </c>
       <c r="BS9" t="n">
-        <v>275.111023540825</v>
+        <v>890.3544933075234</v>
       </c>
       <c r="BT9" t="n">
-        <v>203.9347318424256</v>
+        <v>892.6686924199093</v>
       </c>
       <c r="BU9" t="n">
-        <v>463.6687480765401</v>
+        <v>890.7773893946209</v>
       </c>
       <c r="BV9" t="n">
-        <v>458.8644871299245</v>
+        <v>892.5254197831648</v>
       </c>
       <c r="BW9" t="n">
-        <v>461.6644778517971</v>
+        <v>890.3938738126672</v>
       </c>
       <c r="BX9" t="n">
-        <v>470.9430242458481</v>
+        <v>892.7353908537873</v>
       </c>
       <c r="BY9" t="n">
-        <v>484.2126168267188</v>
+        <v>890.6321815982647</v>
       </c>
       <c r="BZ9" t="n">
-        <v>423.103595549995</v>
+        <v>890.9934866249907</v>
       </c>
       <c r="CA9" t="n">
-        <v>451.1424727431573</v>
+        <v>890.8785680085591</v>
       </c>
       <c r="CB9" t="n">
-        <v>450.1055321692677</v>
+        <v>890.6432937471575</v>
       </c>
       <c r="CC9" t="n">
-        <v>280.2729849967633</v>
+        <v>892.5443422154109</v>
       </c>
       <c r="CD9" t="n">
-        <v>316.1859486212694</v>
+        <v>890.9477813312212</v>
       </c>
       <c r="CE9" t="n">
-        <v>411.8896203656194</v>
+        <v>895.6200617984862</v>
       </c>
       <c r="CF9" t="n">
-        <v>201.0523086680749</v>
+        <v>890.7553018667732</v>
       </c>
       <c r="CG9" t="n">
-        <v>176.6782248077324</v>
+        <v>890.2772391311082</v>
       </c>
       <c r="CH9" t="n">
-        <v>197.4912627868478</v>
+        <v>890.2023048099451</v>
       </c>
       <c r="CI9" t="n">
-        <v>299.3428329466372</v>
+        <v>890.1831453865009</v>
       </c>
       <c r="CJ9" t="n">
-        <v>297.2232716946075</v>
+        <v>893.0196820936868</v>
       </c>
       <c r="CK9" t="n">
-        <v>250.9972947182374</v>
+        <v>892.6132263529316</v>
       </c>
       <c r="CL9" t="n">
-        <v>171.2320480700463</v>
+        <v>643.0182989552793</v>
       </c>
       <c r="CM9" t="n">
-        <v>244.7911763134012</v>
+        <v>646.427221687531</v>
       </c>
       <c r="CN9" t="n">
-        <v>241.3287356510148</v>
+        <v>646.3389908718383</v>
       </c>
       <c r="CO9" t="n">
-        <v>244.9843735972905</v>
+        <v>646.4742986911928</v>
       </c>
       <c r="CP9" t="n">
-        <v>241.4005317748621</v>
+        <v>646.2919334493184</v>
       </c>
       <c r="CQ9" t="n">
-        <v>254.878803125814</v>
+        <v>643.0621396945603</v>
       </c>
       <c r="CR9" t="n">
-        <v>254.2913895238004</v>
+        <v>643.1060247691165</v>
       </c>
       <c r="CS9" t="n">
-        <v>253.8566270999961</v>
+        <v>890.3463307827587</v>
       </c>
       <c r="CT9" t="n">
-        <v>459.1702947490879</v>
+        <v>890.4683802523602</v>
       </c>
       <c r="CU9" t="n">
-        <v>459.0727907924866</v>
+        <v>890.1169514810401</v>
       </c>
       <c r="CV9" t="n">
-        <v>425.3439513159039</v>
+        <v>646.250772008442</v>
       </c>
       <c r="CW9" t="n">
-        <v>454.3209293170943</v>
+        <v>934.9233173529158</v>
       </c>
     </row>
     <row r="10">
@@ -3163,304 +3163,304 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>481.3740692313619</v>
+        <v>1032.544681594848</v>
       </c>
       <c r="C10" t="n">
-        <v>481.2029200620591</v>
+        <v>1034.116321099957</v>
       </c>
       <c r="D10" t="n">
-        <v>493.4204059981676</v>
+        <v>1041.065112435032</v>
       </c>
       <c r="E10" t="n">
-        <v>493.3116352945346</v>
+        <v>1039.659197403994</v>
       </c>
       <c r="F10" t="n">
-        <v>492.877845036049</v>
+        <v>1042.254136376345</v>
       </c>
       <c r="G10" t="n">
-        <v>492.8398027523702</v>
+        <v>1041.967357183936</v>
       </c>
       <c r="H10" t="n">
-        <v>492.5389178048484</v>
+        <v>1022.192656039303</v>
       </c>
       <c r="I10" t="n">
-        <v>505.3427774656331</v>
+        <v>1040.91030622335</v>
       </c>
       <c r="J10" t="n">
-        <v>500.2602588189607</v>
+        <v>1016.674757948937</v>
       </c>
       <c r="K10" t="n">
-        <v>502.5765111329859</v>
+        <v>1017.607753916011</v>
       </c>
       <c r="L10" t="n">
-        <v>501.9256239066611</v>
+        <v>1043.458041707672</v>
       </c>
       <c r="M10" t="n">
-        <v>465.9705344237586</v>
+        <v>1022.498325284937</v>
       </c>
       <c r="N10" t="n">
-        <v>467.5180464556072</v>
+        <v>1018.723199011471</v>
       </c>
       <c r="O10" t="n">
-        <v>468.1588382969989</v>
+        <v>1017.311692666036</v>
       </c>
       <c r="P10" t="n">
-        <v>494.4297923002397</v>
+        <v>997.9645934596978</v>
       </c>
       <c r="Q10" t="n">
-        <v>447.1554199403209</v>
+        <v>997.5541652219642</v>
       </c>
       <c r="R10" t="n">
-        <v>448.9659027328714</v>
+        <v>895.4220495376188</v>
       </c>
       <c r="S10" t="n">
-        <v>443.0916095838814</v>
+        <v>939.7822095844446</v>
       </c>
       <c r="T10" t="n">
-        <v>418.2992824940023</v>
+        <v>998.2065031270915</v>
       </c>
       <c r="U10" t="n">
-        <v>425.8097208189105</v>
+        <v>997.247082108526</v>
       </c>
       <c r="V10" t="n">
-        <v>507.949429748987</v>
+        <v>937.722955018794</v>
       </c>
       <c r="W10" t="n">
-        <v>409.1863954537029</v>
+        <v>997.2435524034363</v>
       </c>
       <c r="X10" t="n">
-        <v>417.8496760650696</v>
+        <v>939.6461200340215</v>
       </c>
       <c r="Y10" t="n">
-        <v>448.2107585527816</v>
+        <v>999.9239249819593</v>
       </c>
       <c r="Z10" t="n">
-        <v>441.1267342773996</v>
+        <v>895.5216142442869</v>
       </c>
       <c r="AA10" t="n">
-        <v>446.0880268856408</v>
+        <v>998.2722535067805</v>
       </c>
       <c r="AB10" t="n">
-        <v>412.1093342210127</v>
+        <v>934.7311681861223</v>
       </c>
       <c r="AC10" t="n">
-        <v>452.6479905625191</v>
+        <v>939.8889355223868</v>
       </c>
       <c r="AD10" t="n">
-        <v>414.6230226123399</v>
+        <v>893.0704300641016</v>
       </c>
       <c r="AE10" t="n">
-        <v>410.8873261957206</v>
+        <v>892.8382015454008</v>
       </c>
       <c r="AF10" t="n">
-        <v>285.7483759288074</v>
+        <v>893.0281756622647</v>
       </c>
       <c r="AG10" t="n">
-        <v>423.7087996634392</v>
+        <v>892.7530926308478</v>
       </c>
       <c r="AH10" t="n">
-        <v>418.6144675698577</v>
+        <v>934.7064058997814</v>
       </c>
       <c r="AI10" t="n">
-        <v>198.0702964792011</v>
+        <v>892.7796972065568</v>
       </c>
       <c r="AJ10" t="n">
-        <v>286.0356524500695</v>
+        <v>646.5944587894304</v>
       </c>
       <c r="AK10" t="n">
-        <v>425.0512106447579</v>
+        <v>892.3817041393424</v>
       </c>
       <c r="AL10" t="n">
-        <v>457.3168670247986</v>
+        <v>892.8190987978287</v>
       </c>
       <c r="AM10" t="n">
-        <v>469.4284507272858</v>
+        <v>646.5568932677812</v>
       </c>
       <c r="AN10" t="n">
-        <v>452.9942016458612</v>
+        <v>890.3745616414624</v>
       </c>
       <c r="AO10" t="n">
-        <v>287.6066570370812</v>
+        <v>644.5899772452583</v>
       </c>
       <c r="AP10" t="n">
-        <v>416.8089591278152</v>
+        <v>646.6878899376655</v>
       </c>
       <c r="AQ10" t="n">
-        <v>412.2364878368156</v>
+        <v>646.3615407036341</v>
       </c>
       <c r="AR10" t="n">
-        <v>410.6634446141057</v>
+        <v>646.7133736955271</v>
       </c>
       <c r="AS10" t="n">
-        <v>456.9140232945576</v>
+        <v>686.3844415783285</v>
       </c>
       <c r="AT10" t="n">
-        <v>337.5392477078975</v>
+        <v>644.3977811879728</v>
       </c>
       <c r="AU10" t="n">
-        <v>324.1639828907005</v>
+        <v>644.1788778312277</v>
       </c>
       <c r="AV10" t="n">
-        <v>205.9244363667606</v>
+        <v>644.6463227645694</v>
       </c>
       <c r="AW10" t="n">
-        <v>414.2410671725296</v>
+        <v>644.3566197470961</v>
       </c>
       <c r="AX10" t="n">
-        <v>405.0350140767178</v>
+        <v>644.4360627311149</v>
       </c>
       <c r="AY10" t="n">
-        <v>409.4077597780985</v>
+        <v>644.5992457609075</v>
       </c>
       <c r="AZ10" t="n">
-        <v>464.2832420347766</v>
+        <v>646.4825553430552</v>
       </c>
       <c r="BA10" t="n">
-        <v>413.2734517325792</v>
+        <v>644.2066927005914</v>
       </c>
       <c r="BB10" t="n">
-        <v>291.7664904081892</v>
+        <v>644.389005308595</v>
       </c>
       <c r="BC10" t="n">
-        <v>194.4711208078839</v>
+        <v>644.7345431400408</v>
       </c>
       <c r="BD10" t="n">
-        <v>193.116709688683</v>
+        <v>644.5330694261853</v>
       </c>
       <c r="BE10" t="n">
-        <v>188.9701508984932</v>
+        <v>644.4448386104925</v>
       </c>
       <c r="BF10" t="n">
-        <v>267.0152401999704</v>
+        <v>646.8240984639758</v>
       </c>
       <c r="BG10" t="n">
-        <v>458.9028303516915</v>
+        <v>644.5110149452148</v>
       </c>
       <c r="BH10" t="n">
-        <v>456.2260721747144</v>
+        <v>644.6404758413219</v>
       </c>
       <c r="BI10" t="n">
-        <v>458.7274947845502</v>
+        <v>644.5465765008328</v>
       </c>
       <c r="BJ10" t="n">
-        <v>416.1648824385792</v>
+        <v>644.4113577283254</v>
       </c>
       <c r="BK10" t="n">
-        <v>413.4630564696756</v>
+        <v>644.3553311490648</v>
       </c>
       <c r="BL10" t="n">
-        <v>411.2278997720683</v>
+        <v>644.4716242867329</v>
       </c>
       <c r="BM10" t="n">
-        <v>290.1026138257334</v>
+        <v>644.4863278189492</v>
       </c>
       <c r="BN10" t="n">
-        <v>193.2703031935559</v>
+        <v>644.7567746087234</v>
       </c>
       <c r="BO10" t="n">
-        <v>284.0181589692821</v>
+        <v>644.5880339062257</v>
       </c>
       <c r="BP10" t="n">
-        <v>187.774923832602</v>
+        <v>644.4528453738023</v>
       </c>
       <c r="BQ10" t="n">
-        <v>244.8974060664625</v>
+        <v>646.8335573413478</v>
       </c>
       <c r="BR10" t="n">
-        <v>275.235863001316</v>
+        <v>649.6481750091392</v>
       </c>
       <c r="BS10" t="n">
-        <v>275.111023540825</v>
+        <v>644.4662594850103</v>
       </c>
       <c r="BT10" t="n">
-        <v>203.9347318424256</v>
+        <v>646.7804585973961</v>
       </c>
       <c r="BU10" t="n">
-        <v>324.6222016157623</v>
+        <v>644.8891555721077</v>
       </c>
       <c r="BV10" t="n">
-        <v>458.8644871299245</v>
+        <v>646.6371859606515</v>
       </c>
       <c r="BW10" t="n">
-        <v>461.6644778517971</v>
+        <v>644.5056399901539</v>
       </c>
       <c r="BX10" t="n">
-        <v>458.5796414405851</v>
+        <v>646.847157031274</v>
       </c>
       <c r="BY10" t="n">
-        <v>484.2126168267188</v>
+        <v>644.7439477757514</v>
       </c>
       <c r="BZ10" t="n">
-        <v>423.103595549995</v>
+        <v>645.1052528024775</v>
       </c>
       <c r="CA10" t="n">
-        <v>451.1424727431573</v>
+        <v>644.990334186046</v>
       </c>
       <c r="CB10" t="n">
-        <v>235.9626648180182</v>
+        <v>644.7550599246442</v>
       </c>
       <c r="CC10" t="n">
-        <v>268.0045073146778</v>
+        <v>646.6561083928975</v>
       </c>
       <c r="CD10" t="n">
-        <v>298.7865321345905</v>
+        <v>645.0595475087081</v>
       </c>
       <c r="CE10" t="n">
-        <v>400.1754550371364</v>
+        <v>649.7318279759729</v>
       </c>
       <c r="CF10" t="n">
-        <v>201.0523086680749</v>
+        <v>644.8670680442599</v>
       </c>
       <c r="CG10" t="n">
-        <v>176.6782248077324</v>
+        <v>400.4036996268052</v>
       </c>
       <c r="CH10" t="n">
-        <v>197.4912627868478</v>
+        <v>644.3140709874318</v>
       </c>
       <c r="CI10" t="n">
-        <v>186.4859766144241</v>
+        <v>649.8659722420125</v>
       </c>
       <c r="CJ10" t="n">
-        <v>285.0096423672804</v>
+        <v>649.8192473613539</v>
       </c>
       <c r="CK10" t="n">
-        <v>238.809326717063</v>
+        <v>646.7249925304184</v>
       </c>
       <c r="CL10" t="n">
-        <v>171.2320480700463</v>
+        <v>397.130065132766</v>
       </c>
       <c r="CM10" t="n">
-        <v>244.7911763134012</v>
+        <v>400.5389878650178</v>
       </c>
       <c r="CN10" t="n">
-        <v>241.3287356510148</v>
+        <v>400.450757049325</v>
       </c>
       <c r="CO10" t="n">
-        <v>244.9843735972905</v>
+        <v>216.0154583599978</v>
       </c>
       <c r="CP10" t="n">
-        <v>241.4005317748621</v>
+        <v>400.4036996268052</v>
       </c>
       <c r="CQ10" t="n">
-        <v>254.878803125814</v>
+        <v>397.1739058720471</v>
       </c>
       <c r="CR10" t="n">
-        <v>242.2226290623029</v>
+        <v>397.2177909466033</v>
       </c>
       <c r="CS10" t="n">
-        <v>241.9050827905325</v>
+        <v>644.4580969602454</v>
       </c>
       <c r="CT10" t="n">
-        <v>320.2098171152653</v>
+        <v>644.5801464298471</v>
       </c>
       <c r="CU10" t="n">
-        <v>459.0727907924866</v>
+        <v>644.2287176585269</v>
       </c>
       <c r="CV10" t="n">
-        <v>414.2204204770765</v>
+        <v>400.3625381859287</v>
       </c>
       <c r="CW10" t="n">
-        <v>454.3209293170943</v>
+        <v>689.0350835304023</v>
       </c>
     </row>
     <row r="11">
@@ -3468,304 +3468,304 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>481.3740692313619</v>
+        <v>1034.106182967596</v>
       </c>
       <c r="C11" t="n">
-        <v>481.2029200620591</v>
+        <v>1034.116321099957</v>
       </c>
       <c r="D11" t="n">
-        <v>493.4204059981676</v>
+        <v>1041.138492596082</v>
       </c>
       <c r="E11" t="n">
-        <v>493.3116352945346</v>
+        <v>1039.659197403994</v>
       </c>
       <c r="F11" t="n">
-        <v>492.877845036049</v>
+        <v>1042.254136376345</v>
       </c>
       <c r="G11" t="n">
-        <v>492.8398027523702</v>
+        <v>1041.967357183936</v>
       </c>
       <c r="H11" t="n">
-        <v>492.5389178048484</v>
+        <v>1022.192656039303</v>
       </c>
       <c r="I11" t="n">
-        <v>505.3427774656331</v>
+        <v>1040.91030622335</v>
       </c>
       <c r="J11" t="n">
-        <v>500.2602588189607</v>
+        <v>1018.718206664664</v>
       </c>
       <c r="K11" t="n">
-        <v>502.5765111329859</v>
+        <v>997.4197856321001</v>
       </c>
       <c r="L11" t="n">
-        <v>463.2619209192903</v>
+        <v>1043.458041707672</v>
       </c>
       <c r="M11" t="n">
-        <v>444.5544129929669</v>
+        <v>1022.498325284937</v>
       </c>
       <c r="N11" t="n">
-        <v>467.5180464556072</v>
+        <v>1018.723199011471</v>
       </c>
       <c r="O11" t="n">
-        <v>468.1588382969989</v>
+        <v>957.6453682876866</v>
       </c>
       <c r="P11" t="n">
-        <v>494.4297923002397</v>
+        <v>997.9645934596978</v>
       </c>
       <c r="Q11" t="n">
-        <v>447.1554199403209</v>
+        <v>997.5541652219642</v>
       </c>
       <c r="R11" t="n">
-        <v>448.9659027328714</v>
+        <v>895.4220495376188</v>
       </c>
       <c r="S11" t="n">
-        <v>443.0916095838814</v>
+        <v>939.7822095844446</v>
       </c>
       <c r="T11" t="n">
-        <v>418.2992824940023</v>
+        <v>998.2065031270915</v>
       </c>
       <c r="U11" t="n">
-        <v>425.8097208189105</v>
+        <v>997.247082108526</v>
       </c>
       <c r="V11" t="n">
-        <v>465.2203119872574</v>
+        <v>935.11740374333</v>
       </c>
       <c r="W11" t="n">
-        <v>409.1863954537029</v>
+        <v>997.2435524034363</v>
       </c>
       <c r="X11" t="n">
-        <v>417.8496760650696</v>
+        <v>895.0509448506755</v>
       </c>
       <c r="Y11" t="n">
-        <v>448.2107585527816</v>
+        <v>999.9239249819593</v>
       </c>
       <c r="Z11" t="n">
-        <v>435.4416763120562</v>
+        <v>892.9160629688229</v>
       </c>
       <c r="AA11" t="n">
-        <v>446.0880268856408</v>
+        <v>998.2722535067805</v>
       </c>
       <c r="AB11" t="n">
-        <v>412.1093342210127</v>
+        <v>934.7311681861223</v>
       </c>
       <c r="AC11" t="n">
-        <v>447.0555706729793</v>
+        <v>937.4830582492016</v>
       </c>
       <c r="AD11" t="n">
-        <v>414.6230226123399</v>
+        <v>893.0704300641016</v>
       </c>
       <c r="AE11" t="n">
-        <v>410.8873261957206</v>
+        <v>892.8382015454008</v>
       </c>
       <c r="AF11" t="n">
-        <v>285.7483759288074</v>
+        <v>646.7557161812645</v>
       </c>
       <c r="AG11" t="n">
-        <v>423.7087996634392</v>
+        <v>892.7530926308478</v>
       </c>
       <c r="AH11" t="n">
-        <v>406.8946994902109</v>
+        <v>892.7290862997877</v>
       </c>
       <c r="AI11" t="n">
-        <v>198.0702964792011</v>
+        <v>892.7796972065568</v>
       </c>
       <c r="AJ11" t="n">
-        <v>286.0356524500695</v>
+        <v>646.5944587894304</v>
       </c>
       <c r="AK11" t="n">
-        <v>413.2933699183653</v>
+        <v>892.3817041393424</v>
       </c>
       <c r="AL11" t="n">
-        <v>457.3168670247986</v>
+        <v>646.6188854460513</v>
       </c>
       <c r="AM11" t="n">
-        <v>457.9376541153799</v>
+        <v>646.5568932677812</v>
       </c>
       <c r="AN11" t="n">
-        <v>336.7016613886052</v>
+        <v>890.3745616414624</v>
       </c>
       <c r="AO11" t="n">
-        <v>192.8545682870178</v>
+        <v>644.5899772452583</v>
       </c>
       <c r="AP11" t="n">
-        <v>416.8089591278152</v>
+        <v>646.6878899376655</v>
       </c>
       <c r="AQ11" t="n">
-        <v>412.2364878368156</v>
+        <v>646.3615407036341</v>
       </c>
       <c r="AR11" t="n">
-        <v>274.6952871608899</v>
+        <v>646.7133736955271</v>
       </c>
       <c r="AS11" t="n">
-        <v>456.9140232945576</v>
+        <v>686.3844415783285</v>
       </c>
       <c r="AT11" t="n">
-        <v>337.5392477078975</v>
+        <v>644.3977811879728</v>
       </c>
       <c r="AU11" t="n">
-        <v>229.3368859921719</v>
+        <v>644.1788778312277</v>
       </c>
       <c r="AV11" t="n">
-        <v>205.9244363667606</v>
+        <v>644.6463227645694</v>
       </c>
       <c r="AW11" t="n">
-        <v>414.2410671725296</v>
+        <v>644.3566197470961</v>
       </c>
       <c r="AX11" t="n">
-        <v>405.0350140767178</v>
+        <v>644.4360627311149</v>
       </c>
       <c r="AY11" t="n">
-        <v>409.4077597780985</v>
+        <v>644.5992457609075</v>
       </c>
       <c r="AZ11" t="n">
-        <v>452.6127053452752</v>
+        <v>646.4825553430552</v>
       </c>
       <c r="BA11" t="n">
-        <v>413.2734517325792</v>
+        <v>644.2066927005914</v>
       </c>
       <c r="BB11" t="n">
-        <v>291.7664904081892</v>
+        <v>644.389005308595</v>
       </c>
       <c r="BC11" t="n">
-        <v>194.4711208078839</v>
+        <v>644.7345431400408</v>
       </c>
       <c r="BD11" t="n">
-        <v>193.116709688683</v>
+        <v>644.5330694261853</v>
       </c>
       <c r="BE11" t="n">
-        <v>188.9701508984932</v>
+        <v>644.4448386104925</v>
       </c>
       <c r="BF11" t="n">
-        <v>267.0152401999704</v>
+        <v>646.8240984639758</v>
       </c>
       <c r="BG11" t="n">
-        <v>411.5594772588414</v>
+        <v>644.5110149452148</v>
       </c>
       <c r="BH11" t="n">
-        <v>456.2260721747144</v>
+        <v>644.6404758413219</v>
       </c>
       <c r="BI11" t="n">
-        <v>458.7274947845502</v>
+        <v>644.5465765008328</v>
       </c>
       <c r="BJ11" t="n">
-        <v>279.6664175724503</v>
+        <v>644.4113577283254</v>
       </c>
       <c r="BK11" t="n">
-        <v>413.4630564696756</v>
+        <v>644.3553311490648</v>
       </c>
       <c r="BL11" t="n">
-        <v>411.2278997720683</v>
+        <v>644.4716242867329</v>
       </c>
       <c r="BM11" t="n">
-        <v>290.1026138257334</v>
+        <v>644.4863278189492</v>
       </c>
       <c r="BN11" t="n">
-        <v>193.2703031935559</v>
+        <v>644.7567746087234</v>
       </c>
       <c r="BO11" t="n">
-        <v>284.0181589692821</v>
+        <v>644.5880339062257</v>
       </c>
       <c r="BP11" t="n">
-        <v>187.774923832602</v>
+        <v>644.4528453738023</v>
       </c>
       <c r="BQ11" t="n">
-        <v>244.8974060664625</v>
+        <v>646.8335573413478</v>
       </c>
       <c r="BR11" t="n">
-        <v>183.5470826662614</v>
+        <v>649.6481750091392</v>
       </c>
       <c r="BS11" t="n">
-        <v>275.111023540825</v>
+        <v>644.4662594850103</v>
       </c>
       <c r="BT11" t="n">
-        <v>203.9347318424256</v>
+        <v>646.7804585973961</v>
       </c>
       <c r="BU11" t="n">
-        <v>324.6222016157623</v>
+        <v>644.8891555721077</v>
       </c>
       <c r="BV11" t="n">
-        <v>303.8525324597775</v>
+        <v>646.6371859606515</v>
       </c>
       <c r="BW11" t="n">
-        <v>461.6644778517971</v>
+        <v>644.5056399901539</v>
       </c>
       <c r="BX11" t="n">
-        <v>458.5796414405851</v>
+        <v>646.847157031274</v>
       </c>
       <c r="BY11" t="n">
-        <v>466.335056911203</v>
+        <v>644.7439477757514</v>
       </c>
       <c r="BZ11" t="n">
-        <v>274.4313083754577</v>
+        <v>645.1052528024775</v>
       </c>
       <c r="CA11" t="n">
-        <v>451.1424727431573</v>
+        <v>644.990334186046</v>
       </c>
       <c r="CB11" t="n">
-        <v>235.9626648180182</v>
+        <v>644.7550599246442</v>
       </c>
       <c r="CC11" t="n">
-        <v>268.0045073146778</v>
+        <v>646.6561083928975</v>
       </c>
       <c r="CD11" t="n">
-        <v>298.7865321345905</v>
+        <v>645.0595475087081</v>
       </c>
       <c r="CE11" t="n">
-        <v>400.1754550371364</v>
+        <v>649.7318279759729</v>
       </c>
       <c r="CF11" t="n">
-        <v>201.0523086680749</v>
+        <v>644.8670680442599</v>
       </c>
       <c r="CG11" t="n">
-        <v>82.19947062650111</v>
+        <v>400.4036996268052</v>
       </c>
       <c r="CH11" t="n">
-        <v>83.98379825002198</v>
+        <v>644.3140709874318</v>
       </c>
       <c r="CI11" t="n">
-        <v>174.3116644881688</v>
+        <v>649.8659722420125</v>
       </c>
       <c r="CJ11" t="n">
-        <v>285.0096423672804</v>
+        <v>649.8192473613539</v>
       </c>
       <c r="CK11" t="n">
-        <v>193.2824032292971</v>
+        <v>400.409659995324</v>
       </c>
       <c r="CL11" t="n">
-        <v>171.2320480700463</v>
+        <v>397.130065132766</v>
       </c>
       <c r="CM11" t="n">
-        <v>244.7911763134012</v>
+        <v>400.5389878650178</v>
       </c>
       <c r="CN11" t="n">
-        <v>241.3287356510148</v>
+        <v>216.0154583599978</v>
       </c>
       <c r="CO11" t="n">
-        <v>244.9843735972905</v>
+        <v>216.0154583599978</v>
       </c>
       <c r="CP11" t="n">
-        <v>86.36543155699449</v>
+        <v>400.4036996268052</v>
       </c>
       <c r="CQ11" t="n">
-        <v>254.878803125814</v>
+        <v>216.0154583599978</v>
       </c>
       <c r="CR11" t="n">
-        <v>242.2226290623029</v>
+        <v>397.2177909466033</v>
       </c>
       <c r="CS11" t="n">
-        <v>241.9050827905325</v>
+        <v>644.4580969602454</v>
       </c>
       <c r="CT11" t="n">
-        <v>320.2098171152653</v>
+        <v>644.5801464298471</v>
       </c>
       <c r="CU11" t="n">
-        <v>459.0727907924866</v>
+        <v>644.2287176585269</v>
       </c>
       <c r="CV11" t="n">
-        <v>414.2204204770765</v>
+        <v>400.3625381859287</v>
       </c>
       <c r="CW11" t="n">
-        <v>454.3209293170943</v>
+        <v>689.0350835304023</v>
       </c>
     </row>
   </sheetData>

</xml_diff>